<commit_message>
Add AI-assisted stamp research engine
</commit_message>
<xml_diff>
--- a/test-fixtures/Stamp-Inventory-Template.xlsx
+++ b/test-fixtures/Stamp-Inventory-Template.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" r:id="Re30f1fab7f1d49d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R88387ac3da9a4405"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per photo" sheetId="3" r:id="Re35787a76f0d46cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress" sheetId="4" r:id="R2b38df67554a451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Raf99a45dc2eb49cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Images" sheetId="6" r:id="R4cc79c0797bb4cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" r:id="Rf18af7fb94b04610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R134a264b0919411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per photo" sheetId="3" r:id="R96e10e3c735447b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress" sheetId="4" r:id="R8f0fb26eaa934913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Rbbb6db3e296849a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Images" sheetId="6" r:id="R1403bb0fb3634f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Summary" sheetId="7" r:id="Rbc8564dc25b540ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -187,14 +188,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="0"/>
     <x:numFmt numFmtId="166" formatCode="\€#,##0.00"/>
     <x:numFmt numFmtId="167" formatCode="0.##"/>
     <x:numFmt numFmtId="168" formatCode="General"/>
+    <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="20">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -296,8 +298,20 @@
       <x:color theme="1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F3864"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -354,8 +368,23 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F3864"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="8">
     <x:border diagonalUp="0" diagonalDown="0"/>
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left style="thin">
@@ -385,6 +414,46 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF1F3864"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="20">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -411,7 +480,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="82">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -592,6 +661,72 @@
     <x:xf numFmtId="164" fontId="17" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="21" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="21" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="21" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="21" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -601,7 +736,7 @@
     <x:cellStyle name="Currency [0]" xfId="18"/>
     <x:cellStyle name="Percent" xfId="19"/>
   </x:cellStyles>
-  <x:dxfs count="9">
+  <x:dxfs count="39">
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -662,6 +797,306 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFFE14D"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFC65911"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF5F497A"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE4DFEC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1086,6 +1521,33 @@
     <x:col min="31" max="31" width="28" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="24" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="24" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="20" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="14" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="12" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="14" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="20" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="14" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="18" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="14" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="24" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="16" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="16" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="16" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="28" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="18" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="18" hidden="0" customWidth="1"/>
+    <x:col min="49" max="49" width="28" hidden="0" customWidth="1"/>
+    <x:col min="50" max="50" width="18" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="18" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="16" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="16" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="30" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="18" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="28" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="28" hidden="0" customWidth="1"/>
+    <x:col min="58" max="58" width="16" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="16" hidden="0" customWidth="1"/>
+    <x:col min="60" max="60" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" hidden="0" customHeight="1">
@@ -1187,6 +1649,87 @@
       </x:c>
       <x:c r="AG1" s="59" t="str">
         <x:v>thumbnail_filename</x:v>
+      </x:c>
+      <x:c r="AH1" s="65" t="str">
+        <x:v>ai_country</x:v>
+      </x:c>
+      <x:c r="AI1" s="65" t="str">
+        <x:v>confidence_country</x:v>
+      </x:c>
+      <x:c r="AJ1" s="65" t="str">
+        <x:v>ai_year</x:v>
+      </x:c>
+      <x:c r="AK1" s="65" t="str">
+        <x:v>confidence_year</x:v>
+      </x:c>
+      <x:c r="AL1" s="65" t="str">
+        <x:v>ai_theme</x:v>
+      </x:c>
+      <x:c r="AM1" s="65" t="str">
+        <x:v>confidence_theme</x:v>
+      </x:c>
+      <x:c r="AN1" s="65" t="str">
+        <x:v>ai_category</x:v>
+      </x:c>
+      <x:c r="AO1" s="65" t="str">
+        <x:v>confidence_category</x:v>
+      </x:c>
+      <x:c r="AP1" s="65" t="str">
+        <x:v>ai_series</x:v>
+      </x:c>
+      <x:c r="AQ1" s="65" t="str">
+        <x:v>confidence_series</x:v>
+      </x:c>
+      <x:c r="AR1" s="65" t="str">
+        <x:v>ai_denomination</x:v>
+      </x:c>
+      <x:c r="AS1" s="65" t="str">
+        <x:v>confidence_denomination</x:v>
+      </x:c>
+      <x:c r="AT1" s="65" t="str">
+        <x:v>visible_text</x:v>
+      </x:c>
+      <x:c r="AU1" s="65" t="str">
+        <x:v>language</x:v>
+      </x:c>
+      <x:c r="AV1" s="65" t="str">
+        <x:v>ai_purpose</x:v>
+      </x:c>
+      <x:c r="AW1" s="65" t="str">
+        <x:v>visual_traits</x:v>
+      </x:c>
+      <x:c r="AX1" s="65" t="str">
+        <x:v>estimated_period</x:v>
+      </x:c>
+      <x:c r="AY1" s="65" t="str">
+        <x:v>dominant_colour</x:v>
+      </x:c>
+      <x:c r="AZ1" s="65" t="str">
+        <x:v>image_quality_score</x:v>
+      </x:c>
+      <x:c r="BA1" s="65" t="str">
+        <x:v>image_quality</x:v>
+      </x:c>
+      <x:c r="BB1" s="65" t="str">
+        <x:v>quality_flags</x:v>
+      </x:c>
+      <x:c r="BC1" s="65" t="str">
+        <x:v>rescan_recommended</x:v>
+      </x:c>
+      <x:c r="BD1" s="65" t="str">
+        <x:v>research_recommendation</x:v>
+      </x:c>
+      <x:c r="BE1" s="65" t="str">
+        <x:v>duplicate_candidate</x:v>
+      </x:c>
+      <x:c r="BF1" s="65" t="str">
+        <x:v>duplicate_similarity</x:v>
+      </x:c>
+      <x:c r="BG1" s="65" t="str">
+        <x:v>overall_confidence</x:v>
+      </x:c>
+      <x:c r="BH1" s="65" t="str">
+        <x:v>research_notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="23.850000381469727" hidden="0">
@@ -1219,6 +1762,15 @@
       <x:c r="Y2" s="49"/>
       <x:c r="Z2" s="49"/>
       <x:c r="AA2" s="49"/>
+      <x:c r="AI2" s="66"/>
+      <x:c r="AK2" s="66"/>
+      <x:c r="AM2" s="66"/>
+      <x:c r="AO2" s="66"/>
+      <x:c r="AQ2" s="66"/>
+      <x:c r="AS2" s="66"/>
+      <x:c r="AZ2" s="66"/>
+      <x:c r="BF2" s="66"/>
+      <x:c r="BG2" s="66"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="18"/>
@@ -1250,6 +1802,15 @@
       <x:c r="Y3" s="49"/>
       <x:c r="Z3" s="49"/>
       <x:c r="AA3" s="49"/>
+      <x:c r="AI3" s="66"/>
+      <x:c r="AK3" s="66"/>
+      <x:c r="AM3" s="66"/>
+      <x:c r="AO3" s="66"/>
+      <x:c r="AQ3" s="66"/>
+      <x:c r="AS3" s="66"/>
+      <x:c r="AZ3" s="66"/>
+      <x:c r="BF3" s="66"/>
+      <x:c r="BG3" s="66"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="18"/>
@@ -1281,6 +1842,15 @@
       <x:c r="Y4" s="49"/>
       <x:c r="Z4" s="49"/>
       <x:c r="AA4" s="49"/>
+      <x:c r="AI4" s="66"/>
+      <x:c r="AK4" s="66"/>
+      <x:c r="AM4" s="66"/>
+      <x:c r="AO4" s="66"/>
+      <x:c r="AQ4" s="66"/>
+      <x:c r="AS4" s="66"/>
+      <x:c r="AZ4" s="66"/>
+      <x:c r="BF4" s="66"/>
+      <x:c r="BG4" s="66"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="18"/>
@@ -1312,6 +1882,15 @@
       <x:c r="Y5" s="49"/>
       <x:c r="Z5" s="49"/>
       <x:c r="AA5" s="49"/>
+      <x:c r="AI5" s="66"/>
+      <x:c r="AK5" s="66"/>
+      <x:c r="AM5" s="66"/>
+      <x:c r="AO5" s="66"/>
+      <x:c r="AQ5" s="66"/>
+      <x:c r="AS5" s="66"/>
+      <x:c r="AZ5" s="66"/>
+      <x:c r="BF5" s="66"/>
+      <x:c r="BG5" s="66"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="18"/>
@@ -1343,6 +1922,15 @@
       <x:c r="Y6" s="49"/>
       <x:c r="Z6" s="49"/>
       <x:c r="AA6" s="49"/>
+      <x:c r="AI6" s="66"/>
+      <x:c r="AK6" s="66"/>
+      <x:c r="AM6" s="66"/>
+      <x:c r="AO6" s="66"/>
+      <x:c r="AQ6" s="66"/>
+      <x:c r="AS6" s="66"/>
+      <x:c r="AZ6" s="66"/>
+      <x:c r="BF6" s="66"/>
+      <x:c r="BG6" s="66"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="18"/>
@@ -1374,6 +1962,15 @@
       <x:c r="Y7" s="49"/>
       <x:c r="Z7" s="49"/>
       <x:c r="AA7" s="49"/>
+      <x:c r="AI7" s="66"/>
+      <x:c r="AK7" s="66"/>
+      <x:c r="AM7" s="66"/>
+      <x:c r="AO7" s="66"/>
+      <x:c r="AQ7" s="66"/>
+      <x:c r="AS7" s="66"/>
+      <x:c r="AZ7" s="66"/>
+      <x:c r="BF7" s="66"/>
+      <x:c r="BG7" s="66"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="18"/>
@@ -1405,6 +2002,15 @@
       <x:c r="Y8" s="49"/>
       <x:c r="Z8" s="49"/>
       <x:c r="AA8" s="49"/>
+      <x:c r="AI8" s="66"/>
+      <x:c r="AK8" s="66"/>
+      <x:c r="AM8" s="66"/>
+      <x:c r="AO8" s="66"/>
+      <x:c r="AQ8" s="66"/>
+      <x:c r="AS8" s="66"/>
+      <x:c r="AZ8" s="66"/>
+      <x:c r="BF8" s="66"/>
+      <x:c r="BG8" s="66"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="18"/>
@@ -1436,6 +2042,15 @@
       <x:c r="Y9" s="49"/>
       <x:c r="Z9" s="49"/>
       <x:c r="AA9" s="49"/>
+      <x:c r="AI9" s="66"/>
+      <x:c r="AK9" s="66"/>
+      <x:c r="AM9" s="66"/>
+      <x:c r="AO9" s="66"/>
+      <x:c r="AQ9" s="66"/>
+      <x:c r="AS9" s="66"/>
+      <x:c r="AZ9" s="66"/>
+      <x:c r="BF9" s="66"/>
+      <x:c r="BG9" s="66"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="18"/>
@@ -1467,6 +2082,15 @@
       <x:c r="Y10" s="49"/>
       <x:c r="Z10" s="49"/>
       <x:c r="AA10" s="49"/>
+      <x:c r="AI10" s="66"/>
+      <x:c r="AK10" s="66"/>
+      <x:c r="AM10" s="66"/>
+      <x:c r="AO10" s="66"/>
+      <x:c r="AQ10" s="66"/>
+      <x:c r="AS10" s="66"/>
+      <x:c r="AZ10" s="66"/>
+      <x:c r="BF10" s="66"/>
+      <x:c r="BG10" s="66"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="18"/>
@@ -1498,6 +2122,15 @@
       <x:c r="Y11" s="49"/>
       <x:c r="Z11" s="49"/>
       <x:c r="AA11" s="49"/>
+      <x:c r="AI11" s="66"/>
+      <x:c r="AK11" s="66"/>
+      <x:c r="AM11" s="66"/>
+      <x:c r="AO11" s="66"/>
+      <x:c r="AQ11" s="66"/>
+      <x:c r="AS11" s="66"/>
+      <x:c r="AZ11" s="66"/>
+      <x:c r="BF11" s="66"/>
+      <x:c r="BG11" s="66"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="18"/>
@@ -1529,6 +2162,15 @@
       <x:c r="Y12" s="49"/>
       <x:c r="Z12" s="49"/>
       <x:c r="AA12" s="49"/>
+      <x:c r="AI12" s="66"/>
+      <x:c r="AK12" s="66"/>
+      <x:c r="AM12" s="66"/>
+      <x:c r="AO12" s="66"/>
+      <x:c r="AQ12" s="66"/>
+      <x:c r="AS12" s="66"/>
+      <x:c r="AZ12" s="66"/>
+      <x:c r="BF12" s="66"/>
+      <x:c r="BG12" s="66"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="18"/>
@@ -1560,6 +2202,15 @@
       <x:c r="Y13" s="49"/>
       <x:c r="Z13" s="49"/>
       <x:c r="AA13" s="49"/>
+      <x:c r="AI13" s="66"/>
+      <x:c r="AK13" s="66"/>
+      <x:c r="AM13" s="66"/>
+      <x:c r="AO13" s="66"/>
+      <x:c r="AQ13" s="66"/>
+      <x:c r="AS13" s="66"/>
+      <x:c r="AZ13" s="66"/>
+      <x:c r="BF13" s="66"/>
+      <x:c r="BG13" s="66"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="18"/>
@@ -1591,6 +2242,15 @@
       <x:c r="Y14" s="49"/>
       <x:c r="Z14" s="49"/>
       <x:c r="AA14" s="49"/>
+      <x:c r="AI14" s="66"/>
+      <x:c r="AK14" s="66"/>
+      <x:c r="AM14" s="66"/>
+      <x:c r="AO14" s="66"/>
+      <x:c r="AQ14" s="66"/>
+      <x:c r="AS14" s="66"/>
+      <x:c r="AZ14" s="66"/>
+      <x:c r="BF14" s="66"/>
+      <x:c r="BG14" s="66"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="18"/>
@@ -1622,6 +2282,15 @@
       <x:c r="Y15" s="49"/>
       <x:c r="Z15" s="49"/>
       <x:c r="AA15" s="49"/>
+      <x:c r="AI15" s="66"/>
+      <x:c r="AK15" s="66"/>
+      <x:c r="AM15" s="66"/>
+      <x:c r="AO15" s="66"/>
+      <x:c r="AQ15" s="66"/>
+      <x:c r="AS15" s="66"/>
+      <x:c r="AZ15" s="66"/>
+      <x:c r="BF15" s="66"/>
+      <x:c r="BG15" s="66"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0">
       <x:c r="A16" s="18"/>
@@ -1653,6 +2322,15 @@
       <x:c r="Y16" s="49"/>
       <x:c r="Z16" s="49"/>
       <x:c r="AA16" s="49"/>
+      <x:c r="AI16" s="66"/>
+      <x:c r="AK16" s="66"/>
+      <x:c r="AM16" s="66"/>
+      <x:c r="AO16" s="66"/>
+      <x:c r="AQ16" s="66"/>
+      <x:c r="AS16" s="66"/>
+      <x:c r="AZ16" s="66"/>
+      <x:c r="BF16" s="66"/>
+      <x:c r="BG16" s="66"/>
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="18"/>
@@ -1684,6 +2362,15 @@
       <x:c r="Y17" s="49"/>
       <x:c r="Z17" s="49"/>
       <x:c r="AA17" s="49"/>
+      <x:c r="AI17" s="66"/>
+      <x:c r="AK17" s="66"/>
+      <x:c r="AM17" s="66"/>
+      <x:c r="AO17" s="66"/>
+      <x:c r="AQ17" s="66"/>
+      <x:c r="AS17" s="66"/>
+      <x:c r="AZ17" s="66"/>
+      <x:c r="BF17" s="66"/>
+      <x:c r="BG17" s="66"/>
     </x:row>
     <x:row r="18" ht="15" hidden="0">
       <x:c r="A18" s="18"/>
@@ -1715,6 +2402,15 @@
       <x:c r="Y18" s="49"/>
       <x:c r="Z18" s="49"/>
       <x:c r="AA18" s="49"/>
+      <x:c r="AI18" s="66"/>
+      <x:c r="AK18" s="66"/>
+      <x:c r="AM18" s="66"/>
+      <x:c r="AO18" s="66"/>
+      <x:c r="AQ18" s="66"/>
+      <x:c r="AS18" s="66"/>
+      <x:c r="AZ18" s="66"/>
+      <x:c r="BF18" s="66"/>
+      <x:c r="BG18" s="66"/>
     </x:row>
     <x:row r="19" ht="15" hidden="0">
       <x:c r="A19" s="18"/>
@@ -1746,6 +2442,15 @@
       <x:c r="Y19" s="49"/>
       <x:c r="Z19" s="49"/>
       <x:c r="AA19" s="49"/>
+      <x:c r="AI19" s="66"/>
+      <x:c r="AK19" s="66"/>
+      <x:c r="AM19" s="66"/>
+      <x:c r="AO19" s="66"/>
+      <x:c r="AQ19" s="66"/>
+      <x:c r="AS19" s="66"/>
+      <x:c r="AZ19" s="66"/>
+      <x:c r="BF19" s="66"/>
+      <x:c r="BG19" s="66"/>
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="18"/>
@@ -1777,6 +2482,15 @@
       <x:c r="Y20" s="49"/>
       <x:c r="Z20" s="49"/>
       <x:c r="AA20" s="49"/>
+      <x:c r="AI20" s="66"/>
+      <x:c r="AK20" s="66"/>
+      <x:c r="AM20" s="66"/>
+      <x:c r="AO20" s="66"/>
+      <x:c r="AQ20" s="66"/>
+      <x:c r="AS20" s="66"/>
+      <x:c r="AZ20" s="66"/>
+      <x:c r="BF20" s="66"/>
+      <x:c r="BG20" s="66"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="18"/>
@@ -1808,6 +2522,15 @@
       <x:c r="Y21" s="49"/>
       <x:c r="Z21" s="49"/>
       <x:c r="AA21" s="49"/>
+      <x:c r="AI21" s="66"/>
+      <x:c r="AK21" s="66"/>
+      <x:c r="AM21" s="66"/>
+      <x:c r="AO21" s="66"/>
+      <x:c r="AQ21" s="66"/>
+      <x:c r="AS21" s="66"/>
+      <x:c r="AZ21" s="66"/>
+      <x:c r="BF21" s="66"/>
+      <x:c r="BG21" s="66"/>
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="18"/>
@@ -1839,6 +2562,15 @@
       <x:c r="Y22" s="49"/>
       <x:c r="Z22" s="49"/>
       <x:c r="AA22" s="49"/>
+      <x:c r="AI22" s="66"/>
+      <x:c r="AK22" s="66"/>
+      <x:c r="AM22" s="66"/>
+      <x:c r="AO22" s="66"/>
+      <x:c r="AQ22" s="66"/>
+      <x:c r="AS22" s="66"/>
+      <x:c r="AZ22" s="66"/>
+      <x:c r="BF22" s="66"/>
+      <x:c r="BG22" s="66"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="18"/>
@@ -1870,6 +2602,15 @@
       <x:c r="Y23" s="49"/>
       <x:c r="Z23" s="49"/>
       <x:c r="AA23" s="49"/>
+      <x:c r="AI23" s="66"/>
+      <x:c r="AK23" s="66"/>
+      <x:c r="AM23" s="66"/>
+      <x:c r="AO23" s="66"/>
+      <x:c r="AQ23" s="66"/>
+      <x:c r="AS23" s="66"/>
+      <x:c r="AZ23" s="66"/>
+      <x:c r="BF23" s="66"/>
+      <x:c r="BG23" s="66"/>
     </x:row>
     <x:row r="24" ht="15" hidden="0">
       <x:c r="A24" s="18"/>
@@ -1901,6 +2642,15 @@
       <x:c r="Y24" s="49"/>
       <x:c r="Z24" s="49"/>
       <x:c r="AA24" s="49"/>
+      <x:c r="AI24" s="66"/>
+      <x:c r="AK24" s="66"/>
+      <x:c r="AM24" s="66"/>
+      <x:c r="AO24" s="66"/>
+      <x:c r="AQ24" s="66"/>
+      <x:c r="AS24" s="66"/>
+      <x:c r="AZ24" s="66"/>
+      <x:c r="BF24" s="66"/>
+      <x:c r="BG24" s="66"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0">
       <x:c r="A25" s="18"/>
@@ -1932,6 +2682,15 @@
       <x:c r="Y25" s="49"/>
       <x:c r="Z25" s="49"/>
       <x:c r="AA25" s="49"/>
+      <x:c r="AI25" s="66"/>
+      <x:c r="AK25" s="66"/>
+      <x:c r="AM25" s="66"/>
+      <x:c r="AO25" s="66"/>
+      <x:c r="AQ25" s="66"/>
+      <x:c r="AS25" s="66"/>
+      <x:c r="AZ25" s="66"/>
+      <x:c r="BF25" s="66"/>
+      <x:c r="BG25" s="66"/>
     </x:row>
     <x:row r="26" ht="15" hidden="0">
       <x:c r="A26" s="18"/>
@@ -1963,6 +2722,15 @@
       <x:c r="Y26" s="49"/>
       <x:c r="Z26" s="49"/>
       <x:c r="AA26" s="49"/>
+      <x:c r="AI26" s="66"/>
+      <x:c r="AK26" s="66"/>
+      <x:c r="AM26" s="66"/>
+      <x:c r="AO26" s="66"/>
+      <x:c r="AQ26" s="66"/>
+      <x:c r="AS26" s="66"/>
+      <x:c r="AZ26" s="66"/>
+      <x:c r="BF26" s="66"/>
+      <x:c r="BG26" s="66"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0">
       <x:c r="A27" s="18"/>
@@ -1994,6 +2762,15 @@
       <x:c r="Y27" s="49"/>
       <x:c r="Z27" s="49"/>
       <x:c r="AA27" s="49"/>
+      <x:c r="AI27" s="66"/>
+      <x:c r="AK27" s="66"/>
+      <x:c r="AM27" s="66"/>
+      <x:c r="AO27" s="66"/>
+      <x:c r="AQ27" s="66"/>
+      <x:c r="AS27" s="66"/>
+      <x:c r="AZ27" s="66"/>
+      <x:c r="BF27" s="66"/>
+      <x:c r="BG27" s="66"/>
     </x:row>
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="18"/>
@@ -2025,6 +2802,15 @@
       <x:c r="Y28" s="49"/>
       <x:c r="Z28" s="49"/>
       <x:c r="AA28" s="49"/>
+      <x:c r="AI28" s="66"/>
+      <x:c r="AK28" s="66"/>
+      <x:c r="AM28" s="66"/>
+      <x:c r="AO28" s="66"/>
+      <x:c r="AQ28" s="66"/>
+      <x:c r="AS28" s="66"/>
+      <x:c r="AZ28" s="66"/>
+      <x:c r="BF28" s="66"/>
+      <x:c r="BG28" s="66"/>
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="18"/>
@@ -2056,6 +2842,15 @@
       <x:c r="Y29" s="49"/>
       <x:c r="Z29" s="49"/>
       <x:c r="AA29" s="49"/>
+      <x:c r="AI29" s="66"/>
+      <x:c r="AK29" s="66"/>
+      <x:c r="AM29" s="66"/>
+      <x:c r="AO29" s="66"/>
+      <x:c r="AQ29" s="66"/>
+      <x:c r="AS29" s="66"/>
+      <x:c r="AZ29" s="66"/>
+      <x:c r="BF29" s="66"/>
+      <x:c r="BG29" s="66"/>
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="18"/>
@@ -2087,6 +2882,15 @@
       <x:c r="Y30" s="49"/>
       <x:c r="Z30" s="49"/>
       <x:c r="AA30" s="49"/>
+      <x:c r="AI30" s="66"/>
+      <x:c r="AK30" s="66"/>
+      <x:c r="AM30" s="66"/>
+      <x:c r="AO30" s="66"/>
+      <x:c r="AQ30" s="66"/>
+      <x:c r="AS30" s="66"/>
+      <x:c r="AZ30" s="66"/>
+      <x:c r="BF30" s="66"/>
+      <x:c r="BG30" s="66"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="18"/>
@@ -2118,6 +2922,15 @@
       <x:c r="Y31" s="49"/>
       <x:c r="Z31" s="49"/>
       <x:c r="AA31" s="49"/>
+      <x:c r="AI31" s="66"/>
+      <x:c r="AK31" s="66"/>
+      <x:c r="AM31" s="66"/>
+      <x:c r="AO31" s="66"/>
+      <x:c r="AQ31" s="66"/>
+      <x:c r="AS31" s="66"/>
+      <x:c r="AZ31" s="66"/>
+      <x:c r="BF31" s="66"/>
+      <x:c r="BG31" s="66"/>
     </x:row>
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="18"/>
@@ -2149,6 +2962,15 @@
       <x:c r="Y32" s="49"/>
       <x:c r="Z32" s="49"/>
       <x:c r="AA32" s="49"/>
+      <x:c r="AI32" s="66"/>
+      <x:c r="AK32" s="66"/>
+      <x:c r="AM32" s="66"/>
+      <x:c r="AO32" s="66"/>
+      <x:c r="AQ32" s="66"/>
+      <x:c r="AS32" s="66"/>
+      <x:c r="AZ32" s="66"/>
+      <x:c r="BF32" s="66"/>
+      <x:c r="BG32" s="66"/>
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="18"/>
@@ -2180,6 +3002,15 @@
       <x:c r="Y33" s="49"/>
       <x:c r="Z33" s="49"/>
       <x:c r="AA33" s="49"/>
+      <x:c r="AI33" s="66"/>
+      <x:c r="AK33" s="66"/>
+      <x:c r="AM33" s="66"/>
+      <x:c r="AO33" s="66"/>
+      <x:c r="AQ33" s="66"/>
+      <x:c r="AS33" s="66"/>
+      <x:c r="AZ33" s="66"/>
+      <x:c r="BF33" s="66"/>
+      <x:c r="BG33" s="66"/>
     </x:row>
     <x:row r="34" ht="15" hidden="0">
       <x:c r="A34" s="18"/>
@@ -2211,6 +3042,15 @@
       <x:c r="Y34" s="49"/>
       <x:c r="Z34" s="49"/>
       <x:c r="AA34" s="49"/>
+      <x:c r="AI34" s="66"/>
+      <x:c r="AK34" s="66"/>
+      <x:c r="AM34" s="66"/>
+      <x:c r="AO34" s="66"/>
+      <x:c r="AQ34" s="66"/>
+      <x:c r="AS34" s="66"/>
+      <x:c r="AZ34" s="66"/>
+      <x:c r="BF34" s="66"/>
+      <x:c r="BG34" s="66"/>
     </x:row>
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="18"/>
@@ -2242,6 +3082,15 @@
       <x:c r="Y35" s="49"/>
       <x:c r="Z35" s="49"/>
       <x:c r="AA35" s="49"/>
+      <x:c r="AI35" s="66"/>
+      <x:c r="AK35" s="66"/>
+      <x:c r="AM35" s="66"/>
+      <x:c r="AO35" s="66"/>
+      <x:c r="AQ35" s="66"/>
+      <x:c r="AS35" s="66"/>
+      <x:c r="AZ35" s="66"/>
+      <x:c r="BF35" s="66"/>
+      <x:c r="BG35" s="66"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="18"/>
@@ -2273,6 +3122,15 @@
       <x:c r="Y36" s="49"/>
       <x:c r="Z36" s="49"/>
       <x:c r="AA36" s="49"/>
+      <x:c r="AI36" s="66"/>
+      <x:c r="AK36" s="66"/>
+      <x:c r="AM36" s="66"/>
+      <x:c r="AO36" s="66"/>
+      <x:c r="AQ36" s="66"/>
+      <x:c r="AS36" s="66"/>
+      <x:c r="AZ36" s="66"/>
+      <x:c r="BF36" s="66"/>
+      <x:c r="BG36" s="66"/>
     </x:row>
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="18"/>
@@ -2304,6 +3162,15 @@
       <x:c r="Y37" s="49"/>
       <x:c r="Z37" s="49"/>
       <x:c r="AA37" s="49"/>
+      <x:c r="AI37" s="66"/>
+      <x:c r="AK37" s="66"/>
+      <x:c r="AM37" s="66"/>
+      <x:c r="AO37" s="66"/>
+      <x:c r="AQ37" s="66"/>
+      <x:c r="AS37" s="66"/>
+      <x:c r="AZ37" s="66"/>
+      <x:c r="BF37" s="66"/>
+      <x:c r="BG37" s="66"/>
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="18"/>
@@ -2335,6 +3202,15 @@
       <x:c r="Y38" s="49"/>
       <x:c r="Z38" s="49"/>
       <x:c r="AA38" s="49"/>
+      <x:c r="AI38" s="66"/>
+      <x:c r="AK38" s="66"/>
+      <x:c r="AM38" s="66"/>
+      <x:c r="AO38" s="66"/>
+      <x:c r="AQ38" s="66"/>
+      <x:c r="AS38" s="66"/>
+      <x:c r="AZ38" s="66"/>
+      <x:c r="BF38" s="66"/>
+      <x:c r="BG38" s="66"/>
     </x:row>
     <x:row r="39" ht="15" hidden="0">
       <x:c r="A39" s="18"/>
@@ -2366,6 +3242,15 @@
       <x:c r="Y39" s="49"/>
       <x:c r="Z39" s="49"/>
       <x:c r="AA39" s="49"/>
+      <x:c r="AI39" s="66"/>
+      <x:c r="AK39" s="66"/>
+      <x:c r="AM39" s="66"/>
+      <x:c r="AO39" s="66"/>
+      <x:c r="AQ39" s="66"/>
+      <x:c r="AS39" s="66"/>
+      <x:c r="AZ39" s="66"/>
+      <x:c r="BF39" s="66"/>
+      <x:c r="BG39" s="66"/>
     </x:row>
     <x:row r="40" ht="15" hidden="0">
       <x:c r="A40" s="18"/>
@@ -2397,6 +3282,15 @@
       <x:c r="Y40" s="49"/>
       <x:c r="Z40" s="49"/>
       <x:c r="AA40" s="49"/>
+      <x:c r="AI40" s="66"/>
+      <x:c r="AK40" s="66"/>
+      <x:c r="AM40" s="66"/>
+      <x:c r="AO40" s="66"/>
+      <x:c r="AQ40" s="66"/>
+      <x:c r="AS40" s="66"/>
+      <x:c r="AZ40" s="66"/>
+      <x:c r="BF40" s="66"/>
+      <x:c r="BG40" s="66"/>
     </x:row>
     <x:row r="41" ht="15" hidden="0">
       <x:c r="A41" s="18"/>
@@ -2428,6 +3322,15 @@
       <x:c r="Y41" s="49"/>
       <x:c r="Z41" s="49"/>
       <x:c r="AA41" s="49"/>
+      <x:c r="AI41" s="66"/>
+      <x:c r="AK41" s="66"/>
+      <x:c r="AM41" s="66"/>
+      <x:c r="AO41" s="66"/>
+      <x:c r="AQ41" s="66"/>
+      <x:c r="AS41" s="66"/>
+      <x:c r="AZ41" s="66"/>
+      <x:c r="BF41" s="66"/>
+      <x:c r="BG41" s="66"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0">
       <x:c r="A42" s="18"/>
@@ -2459,6 +3362,15 @@
       <x:c r="Y42" s="49"/>
       <x:c r="Z42" s="49"/>
       <x:c r="AA42" s="49"/>
+      <x:c r="AI42" s="66"/>
+      <x:c r="AK42" s="66"/>
+      <x:c r="AM42" s="66"/>
+      <x:c r="AO42" s="66"/>
+      <x:c r="AQ42" s="66"/>
+      <x:c r="AS42" s="66"/>
+      <x:c r="AZ42" s="66"/>
+      <x:c r="BF42" s="66"/>
+      <x:c r="BG42" s="66"/>
     </x:row>
     <x:row r="43" ht="15" hidden="0">
       <x:c r="A43" s="18"/>
@@ -2490,6 +3402,15 @@
       <x:c r="Y43" s="49"/>
       <x:c r="Z43" s="49"/>
       <x:c r="AA43" s="49"/>
+      <x:c r="AI43" s="66"/>
+      <x:c r="AK43" s="66"/>
+      <x:c r="AM43" s="66"/>
+      <x:c r="AO43" s="66"/>
+      <x:c r="AQ43" s="66"/>
+      <x:c r="AS43" s="66"/>
+      <x:c r="AZ43" s="66"/>
+      <x:c r="BF43" s="66"/>
+      <x:c r="BG43" s="66"/>
     </x:row>
     <x:row r="44" ht="15" hidden="0">
       <x:c r="A44" s="18"/>
@@ -2521,6 +3442,15 @@
       <x:c r="Y44" s="49"/>
       <x:c r="Z44" s="49"/>
       <x:c r="AA44" s="49"/>
+      <x:c r="AI44" s="66"/>
+      <x:c r="AK44" s="66"/>
+      <x:c r="AM44" s="66"/>
+      <x:c r="AO44" s="66"/>
+      <x:c r="AQ44" s="66"/>
+      <x:c r="AS44" s="66"/>
+      <x:c r="AZ44" s="66"/>
+      <x:c r="BF44" s="66"/>
+      <x:c r="BG44" s="66"/>
     </x:row>
     <x:row r="45" ht="15" hidden="0">
       <x:c r="A45" s="18"/>
@@ -2552,6 +3482,15 @@
       <x:c r="Y45" s="49"/>
       <x:c r="Z45" s="49"/>
       <x:c r="AA45" s="49"/>
+      <x:c r="AI45" s="66"/>
+      <x:c r="AK45" s="66"/>
+      <x:c r="AM45" s="66"/>
+      <x:c r="AO45" s="66"/>
+      <x:c r="AQ45" s="66"/>
+      <x:c r="AS45" s="66"/>
+      <x:c r="AZ45" s="66"/>
+      <x:c r="BF45" s="66"/>
+      <x:c r="BG45" s="66"/>
     </x:row>
     <x:row r="46" ht="15" hidden="0">
       <x:c r="A46" s="18"/>
@@ -2583,6 +3522,15 @@
       <x:c r="Y46" s="49"/>
       <x:c r="Z46" s="49"/>
       <x:c r="AA46" s="49"/>
+      <x:c r="AI46" s="66"/>
+      <x:c r="AK46" s="66"/>
+      <x:c r="AM46" s="66"/>
+      <x:c r="AO46" s="66"/>
+      <x:c r="AQ46" s="66"/>
+      <x:c r="AS46" s="66"/>
+      <x:c r="AZ46" s="66"/>
+      <x:c r="BF46" s="66"/>
+      <x:c r="BG46" s="66"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0">
       <x:c r="A47" s="18"/>
@@ -2614,6 +3562,15 @@
       <x:c r="Y47" s="49"/>
       <x:c r="Z47" s="49"/>
       <x:c r="AA47" s="49"/>
+      <x:c r="AI47" s="66"/>
+      <x:c r="AK47" s="66"/>
+      <x:c r="AM47" s="66"/>
+      <x:c r="AO47" s="66"/>
+      <x:c r="AQ47" s="66"/>
+      <x:c r="AS47" s="66"/>
+      <x:c r="AZ47" s="66"/>
+      <x:c r="BF47" s="66"/>
+      <x:c r="BG47" s="66"/>
     </x:row>
     <x:row r="48" ht="15" hidden="0">
       <x:c r="A48" s="18"/>
@@ -2645,6 +3602,15 @@
       <x:c r="Y48" s="49"/>
       <x:c r="Z48" s="49"/>
       <x:c r="AA48" s="49"/>
+      <x:c r="AI48" s="66"/>
+      <x:c r="AK48" s="66"/>
+      <x:c r="AM48" s="66"/>
+      <x:c r="AO48" s="66"/>
+      <x:c r="AQ48" s="66"/>
+      <x:c r="AS48" s="66"/>
+      <x:c r="AZ48" s="66"/>
+      <x:c r="BF48" s="66"/>
+      <x:c r="BG48" s="66"/>
     </x:row>
     <x:row r="49" ht="15" hidden="0">
       <x:c r="A49" s="18"/>
@@ -2676,6 +3642,15 @@
       <x:c r="Y49" s="49"/>
       <x:c r="Z49" s="49"/>
       <x:c r="AA49" s="49"/>
+      <x:c r="AI49" s="66"/>
+      <x:c r="AK49" s="66"/>
+      <x:c r="AM49" s="66"/>
+      <x:c r="AO49" s="66"/>
+      <x:c r="AQ49" s="66"/>
+      <x:c r="AS49" s="66"/>
+      <x:c r="AZ49" s="66"/>
+      <x:c r="BF49" s="66"/>
+      <x:c r="BG49" s="66"/>
     </x:row>
     <x:row r="50" ht="15" hidden="0">
       <x:c r="A50" s="18"/>
@@ -2707,6 +3682,15 @@
       <x:c r="Y50" s="49"/>
       <x:c r="Z50" s="49"/>
       <x:c r="AA50" s="49"/>
+      <x:c r="AI50" s="66"/>
+      <x:c r="AK50" s="66"/>
+      <x:c r="AM50" s="66"/>
+      <x:c r="AO50" s="66"/>
+      <x:c r="AQ50" s="66"/>
+      <x:c r="AS50" s="66"/>
+      <x:c r="AZ50" s="66"/>
+      <x:c r="BF50" s="66"/>
+      <x:c r="BG50" s="66"/>
     </x:row>
     <x:row r="51" ht="15" hidden="0">
       <x:c r="A51" s="18"/>
@@ -2738,6 +3722,15 @@
       <x:c r="Y51" s="49"/>
       <x:c r="Z51" s="49"/>
       <x:c r="AA51" s="49"/>
+      <x:c r="AI51" s="66"/>
+      <x:c r="AK51" s="66"/>
+      <x:c r="AM51" s="66"/>
+      <x:c r="AO51" s="66"/>
+      <x:c r="AQ51" s="66"/>
+      <x:c r="AS51" s="66"/>
+      <x:c r="AZ51" s="66"/>
+      <x:c r="BF51" s="66"/>
+      <x:c r="BG51" s="66"/>
     </x:row>
     <x:row r="52" ht="15" hidden="0">
       <x:c r="A52" s="18"/>
@@ -2769,6 +3762,15 @@
       <x:c r="Y52" s="49"/>
       <x:c r="Z52" s="49"/>
       <x:c r="AA52" s="49"/>
+      <x:c r="AI52" s="66"/>
+      <x:c r="AK52" s="66"/>
+      <x:c r="AM52" s="66"/>
+      <x:c r="AO52" s="66"/>
+      <x:c r="AQ52" s="66"/>
+      <x:c r="AS52" s="66"/>
+      <x:c r="AZ52" s="66"/>
+      <x:c r="BF52" s="66"/>
+      <x:c r="BG52" s="66"/>
     </x:row>
     <x:row r="53" ht="15" hidden="0">
       <x:c r="A53" s="18"/>
@@ -2800,6 +3802,15 @@
       <x:c r="Y53" s="49"/>
       <x:c r="Z53" s="49"/>
       <x:c r="AA53" s="49"/>
+      <x:c r="AI53" s="66"/>
+      <x:c r="AK53" s="66"/>
+      <x:c r="AM53" s="66"/>
+      <x:c r="AO53" s="66"/>
+      <x:c r="AQ53" s="66"/>
+      <x:c r="AS53" s="66"/>
+      <x:c r="AZ53" s="66"/>
+      <x:c r="BF53" s="66"/>
+      <x:c r="BG53" s="66"/>
     </x:row>
     <x:row r="54" ht="15" hidden="0">
       <x:c r="A54" s="18"/>
@@ -2831,6 +3842,15 @@
       <x:c r="Y54" s="49"/>
       <x:c r="Z54" s="49"/>
       <x:c r="AA54" s="49"/>
+      <x:c r="AI54" s="66"/>
+      <x:c r="AK54" s="66"/>
+      <x:c r="AM54" s="66"/>
+      <x:c r="AO54" s="66"/>
+      <x:c r="AQ54" s="66"/>
+      <x:c r="AS54" s="66"/>
+      <x:c r="AZ54" s="66"/>
+      <x:c r="BF54" s="66"/>
+      <x:c r="BG54" s="66"/>
     </x:row>
     <x:row r="55" ht="15" hidden="0">
       <x:c r="A55" s="18"/>
@@ -2862,6 +3882,15 @@
       <x:c r="Y55" s="49"/>
       <x:c r="Z55" s="49"/>
       <x:c r="AA55" s="49"/>
+      <x:c r="AI55" s="66"/>
+      <x:c r="AK55" s="66"/>
+      <x:c r="AM55" s="66"/>
+      <x:c r="AO55" s="66"/>
+      <x:c r="AQ55" s="66"/>
+      <x:c r="AS55" s="66"/>
+      <x:c r="AZ55" s="66"/>
+      <x:c r="BF55" s="66"/>
+      <x:c r="BG55" s="66"/>
     </x:row>
     <x:row r="56" ht="15" hidden="0">
       <x:c r="A56" s="18"/>
@@ -2893,6 +3922,15 @@
       <x:c r="Y56" s="49"/>
       <x:c r="Z56" s="49"/>
       <x:c r="AA56" s="49"/>
+      <x:c r="AI56" s="66"/>
+      <x:c r="AK56" s="66"/>
+      <x:c r="AM56" s="66"/>
+      <x:c r="AO56" s="66"/>
+      <x:c r="AQ56" s="66"/>
+      <x:c r="AS56" s="66"/>
+      <x:c r="AZ56" s="66"/>
+      <x:c r="BF56" s="66"/>
+      <x:c r="BG56" s="66"/>
     </x:row>
     <x:row r="57" ht="15" hidden="0">
       <x:c r="A57" s="18"/>
@@ -2924,6 +3962,15 @@
       <x:c r="Y57" s="49"/>
       <x:c r="Z57" s="49"/>
       <x:c r="AA57" s="49"/>
+      <x:c r="AI57" s="66"/>
+      <x:c r="AK57" s="66"/>
+      <x:c r="AM57" s="66"/>
+      <x:c r="AO57" s="66"/>
+      <x:c r="AQ57" s="66"/>
+      <x:c r="AS57" s="66"/>
+      <x:c r="AZ57" s="66"/>
+      <x:c r="BF57" s="66"/>
+      <x:c r="BG57" s="66"/>
     </x:row>
     <x:row r="58" ht="15" hidden="0">
       <x:c r="A58" s="18"/>
@@ -2955,6 +4002,15 @@
       <x:c r="Y58" s="49"/>
       <x:c r="Z58" s="49"/>
       <x:c r="AA58" s="49"/>
+      <x:c r="AI58" s="66"/>
+      <x:c r="AK58" s="66"/>
+      <x:c r="AM58" s="66"/>
+      <x:c r="AO58" s="66"/>
+      <x:c r="AQ58" s="66"/>
+      <x:c r="AS58" s="66"/>
+      <x:c r="AZ58" s="66"/>
+      <x:c r="BF58" s="66"/>
+      <x:c r="BG58" s="66"/>
     </x:row>
     <x:row r="59" ht="15" hidden="0">
       <x:c r="A59" s="18"/>
@@ -2986,6 +4042,15 @@
       <x:c r="Y59" s="49"/>
       <x:c r="Z59" s="49"/>
       <x:c r="AA59" s="49"/>
+      <x:c r="AI59" s="66"/>
+      <x:c r="AK59" s="66"/>
+      <x:c r="AM59" s="66"/>
+      <x:c r="AO59" s="66"/>
+      <x:c r="AQ59" s="66"/>
+      <x:c r="AS59" s="66"/>
+      <x:c r="AZ59" s="66"/>
+      <x:c r="BF59" s="66"/>
+      <x:c r="BG59" s="66"/>
     </x:row>
     <x:row r="60" ht="15" hidden="0">
       <x:c r="A60" s="18"/>
@@ -3017,6 +4082,15 @@
       <x:c r="Y60" s="49"/>
       <x:c r="Z60" s="49"/>
       <x:c r="AA60" s="49"/>
+      <x:c r="AI60" s="66"/>
+      <x:c r="AK60" s="66"/>
+      <x:c r="AM60" s="66"/>
+      <x:c r="AO60" s="66"/>
+      <x:c r="AQ60" s="66"/>
+      <x:c r="AS60" s="66"/>
+      <x:c r="AZ60" s="66"/>
+      <x:c r="BF60" s="66"/>
+      <x:c r="BG60" s="66"/>
     </x:row>
     <x:row r="61" ht="15" hidden="0">
       <x:c r="A61" s="18"/>
@@ -3048,6 +4122,15 @@
       <x:c r="Y61" s="49"/>
       <x:c r="Z61" s="49"/>
       <x:c r="AA61" s="49"/>
+      <x:c r="AI61" s="66"/>
+      <x:c r="AK61" s="66"/>
+      <x:c r="AM61" s="66"/>
+      <x:c r="AO61" s="66"/>
+      <x:c r="AQ61" s="66"/>
+      <x:c r="AS61" s="66"/>
+      <x:c r="AZ61" s="66"/>
+      <x:c r="BF61" s="66"/>
+      <x:c r="BG61" s="66"/>
     </x:row>
     <x:row r="62" ht="15" hidden="0">
       <x:c r="A62" s="18"/>
@@ -3079,6 +4162,15 @@
       <x:c r="Y62" s="49"/>
       <x:c r="Z62" s="49"/>
       <x:c r="AA62" s="49"/>
+      <x:c r="AI62" s="66"/>
+      <x:c r="AK62" s="66"/>
+      <x:c r="AM62" s="66"/>
+      <x:c r="AO62" s="66"/>
+      <x:c r="AQ62" s="66"/>
+      <x:c r="AS62" s="66"/>
+      <x:c r="AZ62" s="66"/>
+      <x:c r="BF62" s="66"/>
+      <x:c r="BG62" s="66"/>
     </x:row>
     <x:row r="63" ht="15" hidden="0">
       <x:c r="A63" s="18"/>
@@ -3110,6 +4202,15 @@
       <x:c r="Y63" s="49"/>
       <x:c r="Z63" s="49"/>
       <x:c r="AA63" s="49"/>
+      <x:c r="AI63" s="66"/>
+      <x:c r="AK63" s="66"/>
+      <x:c r="AM63" s="66"/>
+      <x:c r="AO63" s="66"/>
+      <x:c r="AQ63" s="66"/>
+      <x:c r="AS63" s="66"/>
+      <x:c r="AZ63" s="66"/>
+      <x:c r="BF63" s="66"/>
+      <x:c r="BG63" s="66"/>
     </x:row>
     <x:row r="64" ht="15" hidden="0">
       <x:c r="A64" s="18"/>
@@ -3141,6 +4242,15 @@
       <x:c r="Y64" s="49"/>
       <x:c r="Z64" s="49"/>
       <x:c r="AA64" s="49"/>
+      <x:c r="AI64" s="66"/>
+      <x:c r="AK64" s="66"/>
+      <x:c r="AM64" s="66"/>
+      <x:c r="AO64" s="66"/>
+      <x:c r="AQ64" s="66"/>
+      <x:c r="AS64" s="66"/>
+      <x:c r="AZ64" s="66"/>
+      <x:c r="BF64" s="66"/>
+      <x:c r="BG64" s="66"/>
     </x:row>
     <x:row r="65" ht="15" hidden="0">
       <x:c r="A65" s="18"/>
@@ -3172,6 +4282,15 @@
       <x:c r="Y65" s="49"/>
       <x:c r="Z65" s="49"/>
       <x:c r="AA65" s="49"/>
+      <x:c r="AI65" s="66"/>
+      <x:c r="AK65" s="66"/>
+      <x:c r="AM65" s="66"/>
+      <x:c r="AO65" s="66"/>
+      <x:c r="AQ65" s="66"/>
+      <x:c r="AS65" s="66"/>
+      <x:c r="AZ65" s="66"/>
+      <x:c r="BF65" s="66"/>
+      <x:c r="BG65" s="66"/>
     </x:row>
     <x:row r="66" ht="15" hidden="0">
       <x:c r="A66" s="18"/>
@@ -3203,6 +4322,15 @@
       <x:c r="Y66" s="49"/>
       <x:c r="Z66" s="49"/>
       <x:c r="AA66" s="49"/>
+      <x:c r="AI66" s="66"/>
+      <x:c r="AK66" s="66"/>
+      <x:c r="AM66" s="66"/>
+      <x:c r="AO66" s="66"/>
+      <x:c r="AQ66" s="66"/>
+      <x:c r="AS66" s="66"/>
+      <x:c r="AZ66" s="66"/>
+      <x:c r="BF66" s="66"/>
+      <x:c r="BG66" s="66"/>
     </x:row>
     <x:row r="67" ht="15" hidden="0">
       <x:c r="A67" s="18"/>
@@ -3234,6 +4362,15 @@
       <x:c r="Y67" s="49"/>
       <x:c r="Z67" s="49"/>
       <x:c r="AA67" s="49"/>
+      <x:c r="AI67" s="66"/>
+      <x:c r="AK67" s="66"/>
+      <x:c r="AM67" s="66"/>
+      <x:c r="AO67" s="66"/>
+      <x:c r="AQ67" s="66"/>
+      <x:c r="AS67" s="66"/>
+      <x:c r="AZ67" s="66"/>
+      <x:c r="BF67" s="66"/>
+      <x:c r="BG67" s="66"/>
     </x:row>
     <x:row r="68" ht="15" hidden="0">
       <x:c r="A68" s="18"/>
@@ -3265,6 +4402,15 @@
       <x:c r="Y68" s="49"/>
       <x:c r="Z68" s="49"/>
       <x:c r="AA68" s="49"/>
+      <x:c r="AI68" s="66"/>
+      <x:c r="AK68" s="66"/>
+      <x:c r="AM68" s="66"/>
+      <x:c r="AO68" s="66"/>
+      <x:c r="AQ68" s="66"/>
+      <x:c r="AS68" s="66"/>
+      <x:c r="AZ68" s="66"/>
+      <x:c r="BF68" s="66"/>
+      <x:c r="BG68" s="66"/>
     </x:row>
     <x:row r="69" ht="15" hidden="0">
       <x:c r="A69" s="18"/>
@@ -3296,6 +4442,15 @@
       <x:c r="Y69" s="49"/>
       <x:c r="Z69" s="49"/>
       <x:c r="AA69" s="49"/>
+      <x:c r="AI69" s="66"/>
+      <x:c r="AK69" s="66"/>
+      <x:c r="AM69" s="66"/>
+      <x:c r="AO69" s="66"/>
+      <x:c r="AQ69" s="66"/>
+      <x:c r="AS69" s="66"/>
+      <x:c r="AZ69" s="66"/>
+      <x:c r="BF69" s="66"/>
+      <x:c r="BG69" s="66"/>
     </x:row>
     <x:row r="70" ht="15" hidden="0">
       <x:c r="A70" s="18"/>
@@ -3327,6 +4482,15 @@
       <x:c r="Y70" s="49"/>
       <x:c r="Z70" s="49"/>
       <x:c r="AA70" s="49"/>
+      <x:c r="AI70" s="66"/>
+      <x:c r="AK70" s="66"/>
+      <x:c r="AM70" s="66"/>
+      <x:c r="AO70" s="66"/>
+      <x:c r="AQ70" s="66"/>
+      <x:c r="AS70" s="66"/>
+      <x:c r="AZ70" s="66"/>
+      <x:c r="BF70" s="66"/>
+      <x:c r="BG70" s="66"/>
     </x:row>
     <x:row r="71" ht="15" hidden="0">
       <x:c r="A71" s="18"/>
@@ -3358,6 +4522,15 @@
       <x:c r="Y71" s="49"/>
       <x:c r="Z71" s="49"/>
       <x:c r="AA71" s="49"/>
+      <x:c r="AI71" s="66"/>
+      <x:c r="AK71" s="66"/>
+      <x:c r="AM71" s="66"/>
+      <x:c r="AO71" s="66"/>
+      <x:c r="AQ71" s="66"/>
+      <x:c r="AS71" s="66"/>
+      <x:c r="AZ71" s="66"/>
+      <x:c r="BF71" s="66"/>
+      <x:c r="BG71" s="66"/>
     </x:row>
     <x:row r="72" ht="15" hidden="0">
       <x:c r="A72" s="18"/>
@@ -3389,6 +4562,15 @@
       <x:c r="Y72" s="49"/>
       <x:c r="Z72" s="49"/>
       <x:c r="AA72" s="49"/>
+      <x:c r="AI72" s="66"/>
+      <x:c r="AK72" s="66"/>
+      <x:c r="AM72" s="66"/>
+      <x:c r="AO72" s="66"/>
+      <x:c r="AQ72" s="66"/>
+      <x:c r="AS72" s="66"/>
+      <x:c r="AZ72" s="66"/>
+      <x:c r="BF72" s="66"/>
+      <x:c r="BG72" s="66"/>
     </x:row>
     <x:row r="73" ht="15" hidden="0">
       <x:c r="A73" s="18"/>
@@ -3420,6 +4602,15 @@
       <x:c r="Y73" s="49"/>
       <x:c r="Z73" s="49"/>
       <x:c r="AA73" s="49"/>
+      <x:c r="AI73" s="66"/>
+      <x:c r="AK73" s="66"/>
+      <x:c r="AM73" s="66"/>
+      <x:c r="AO73" s="66"/>
+      <x:c r="AQ73" s="66"/>
+      <x:c r="AS73" s="66"/>
+      <x:c r="AZ73" s="66"/>
+      <x:c r="BF73" s="66"/>
+      <x:c r="BG73" s="66"/>
     </x:row>
     <x:row r="74" ht="15" hidden="0">
       <x:c r="A74" s="18"/>
@@ -3451,6 +4642,15 @@
       <x:c r="Y74" s="49"/>
       <x:c r="Z74" s="49"/>
       <x:c r="AA74" s="49"/>
+      <x:c r="AI74" s="66"/>
+      <x:c r="AK74" s="66"/>
+      <x:c r="AM74" s="66"/>
+      <x:c r="AO74" s="66"/>
+      <x:c r="AQ74" s="66"/>
+      <x:c r="AS74" s="66"/>
+      <x:c r="AZ74" s="66"/>
+      <x:c r="BF74" s="66"/>
+      <x:c r="BG74" s="66"/>
     </x:row>
     <x:row r="75" ht="15" hidden="0">
       <x:c r="A75" s="18"/>
@@ -3482,6 +4682,15 @@
       <x:c r="Y75" s="49"/>
       <x:c r="Z75" s="49"/>
       <x:c r="AA75" s="49"/>
+      <x:c r="AI75" s="66"/>
+      <x:c r="AK75" s="66"/>
+      <x:c r="AM75" s="66"/>
+      <x:c r="AO75" s="66"/>
+      <x:c r="AQ75" s="66"/>
+      <x:c r="AS75" s="66"/>
+      <x:c r="AZ75" s="66"/>
+      <x:c r="BF75" s="66"/>
+      <x:c r="BG75" s="66"/>
     </x:row>
     <x:row r="76" ht="15" hidden="0">
       <x:c r="A76" s="18"/>
@@ -3513,6 +4722,15 @@
       <x:c r="Y76" s="49"/>
       <x:c r="Z76" s="49"/>
       <x:c r="AA76" s="49"/>
+      <x:c r="AI76" s="66"/>
+      <x:c r="AK76" s="66"/>
+      <x:c r="AM76" s="66"/>
+      <x:c r="AO76" s="66"/>
+      <x:c r="AQ76" s="66"/>
+      <x:c r="AS76" s="66"/>
+      <x:c r="AZ76" s="66"/>
+      <x:c r="BF76" s="66"/>
+      <x:c r="BG76" s="66"/>
     </x:row>
     <x:row r="77" ht="15" hidden="0">
       <x:c r="A77" s="18"/>
@@ -3544,6 +4762,15 @@
       <x:c r="Y77" s="49"/>
       <x:c r="Z77" s="49"/>
       <x:c r="AA77" s="49"/>
+      <x:c r="AI77" s="66"/>
+      <x:c r="AK77" s="66"/>
+      <x:c r="AM77" s="66"/>
+      <x:c r="AO77" s="66"/>
+      <x:c r="AQ77" s="66"/>
+      <x:c r="AS77" s="66"/>
+      <x:c r="AZ77" s="66"/>
+      <x:c r="BF77" s="66"/>
+      <x:c r="BG77" s="66"/>
     </x:row>
     <x:row r="78" ht="15" hidden="0">
       <x:c r="A78" s="18"/>
@@ -3575,6 +4802,15 @@
       <x:c r="Y78" s="49"/>
       <x:c r="Z78" s="49"/>
       <x:c r="AA78" s="49"/>
+      <x:c r="AI78" s="66"/>
+      <x:c r="AK78" s="66"/>
+      <x:c r="AM78" s="66"/>
+      <x:c r="AO78" s="66"/>
+      <x:c r="AQ78" s="66"/>
+      <x:c r="AS78" s="66"/>
+      <x:c r="AZ78" s="66"/>
+      <x:c r="BF78" s="66"/>
+      <x:c r="BG78" s="66"/>
     </x:row>
     <x:row r="79" ht="15" hidden="0">
       <x:c r="A79" s="18"/>
@@ -3606,6 +4842,15 @@
       <x:c r="Y79" s="49"/>
       <x:c r="Z79" s="49"/>
       <x:c r="AA79" s="49"/>
+      <x:c r="AI79" s="66"/>
+      <x:c r="AK79" s="66"/>
+      <x:c r="AM79" s="66"/>
+      <x:c r="AO79" s="66"/>
+      <x:c r="AQ79" s="66"/>
+      <x:c r="AS79" s="66"/>
+      <x:c r="AZ79" s="66"/>
+      <x:c r="BF79" s="66"/>
+      <x:c r="BG79" s="66"/>
     </x:row>
     <x:row r="80" ht="15" hidden="0">
       <x:c r="A80" s="18"/>
@@ -3637,6 +4882,15 @@
       <x:c r="Y80" s="49"/>
       <x:c r="Z80" s="49"/>
       <x:c r="AA80" s="49"/>
+      <x:c r="AI80" s="66"/>
+      <x:c r="AK80" s="66"/>
+      <x:c r="AM80" s="66"/>
+      <x:c r="AO80" s="66"/>
+      <x:c r="AQ80" s="66"/>
+      <x:c r="AS80" s="66"/>
+      <x:c r="AZ80" s="66"/>
+      <x:c r="BF80" s="66"/>
+      <x:c r="BG80" s="66"/>
     </x:row>
     <x:row r="81" ht="15" hidden="0">
       <x:c r="A81" s="18"/>
@@ -3668,6 +4922,15 @@
       <x:c r="Y81" s="49"/>
       <x:c r="Z81" s="49"/>
       <x:c r="AA81" s="49"/>
+      <x:c r="AI81" s="66"/>
+      <x:c r="AK81" s="66"/>
+      <x:c r="AM81" s="66"/>
+      <x:c r="AO81" s="66"/>
+      <x:c r="AQ81" s="66"/>
+      <x:c r="AS81" s="66"/>
+      <x:c r="AZ81" s="66"/>
+      <x:c r="BF81" s="66"/>
+      <x:c r="BG81" s="66"/>
     </x:row>
     <x:row r="82" ht="15" hidden="0">
       <x:c r="A82" s="18"/>
@@ -3699,6 +4962,15 @@
       <x:c r="Y82" s="49"/>
       <x:c r="Z82" s="49"/>
       <x:c r="AA82" s="49"/>
+      <x:c r="AI82" s="66"/>
+      <x:c r="AK82" s="66"/>
+      <x:c r="AM82" s="66"/>
+      <x:c r="AO82" s="66"/>
+      <x:c r="AQ82" s="66"/>
+      <x:c r="AS82" s="66"/>
+      <x:c r="AZ82" s="66"/>
+      <x:c r="BF82" s="66"/>
+      <x:c r="BG82" s="66"/>
     </x:row>
     <x:row r="83" ht="15" hidden="0">
       <x:c r="A83" s="18"/>
@@ -3730,6 +5002,15 @@
       <x:c r="Y83" s="49"/>
       <x:c r="Z83" s="49"/>
       <x:c r="AA83" s="49"/>
+      <x:c r="AI83" s="66"/>
+      <x:c r="AK83" s="66"/>
+      <x:c r="AM83" s="66"/>
+      <x:c r="AO83" s="66"/>
+      <x:c r="AQ83" s="66"/>
+      <x:c r="AS83" s="66"/>
+      <x:c r="AZ83" s="66"/>
+      <x:c r="BF83" s="66"/>
+      <x:c r="BG83" s="66"/>
     </x:row>
     <x:row r="84" ht="15" hidden="0">
       <x:c r="A84" s="18"/>
@@ -3761,6 +5042,15 @@
       <x:c r="Y84" s="49"/>
       <x:c r="Z84" s="49"/>
       <x:c r="AA84" s="49"/>
+      <x:c r="AI84" s="66"/>
+      <x:c r="AK84" s="66"/>
+      <x:c r="AM84" s="66"/>
+      <x:c r="AO84" s="66"/>
+      <x:c r="AQ84" s="66"/>
+      <x:c r="AS84" s="66"/>
+      <x:c r="AZ84" s="66"/>
+      <x:c r="BF84" s="66"/>
+      <x:c r="BG84" s="66"/>
     </x:row>
     <x:row r="85" ht="15" hidden="0">
       <x:c r="A85" s="18"/>
@@ -3792,6 +5082,15 @@
       <x:c r="Y85" s="49"/>
       <x:c r="Z85" s="49"/>
       <x:c r="AA85" s="49"/>
+      <x:c r="AI85" s="66"/>
+      <x:c r="AK85" s="66"/>
+      <x:c r="AM85" s="66"/>
+      <x:c r="AO85" s="66"/>
+      <x:c r="AQ85" s="66"/>
+      <x:c r="AS85" s="66"/>
+      <x:c r="AZ85" s="66"/>
+      <x:c r="BF85" s="66"/>
+      <x:c r="BG85" s="66"/>
     </x:row>
     <x:row r="86" ht="15" hidden="0">
       <x:c r="A86" s="18"/>
@@ -3823,6 +5122,15 @@
       <x:c r="Y86" s="49"/>
       <x:c r="Z86" s="49"/>
       <x:c r="AA86" s="49"/>
+      <x:c r="AI86" s="66"/>
+      <x:c r="AK86" s="66"/>
+      <x:c r="AM86" s="66"/>
+      <x:c r="AO86" s="66"/>
+      <x:c r="AQ86" s="66"/>
+      <x:c r="AS86" s="66"/>
+      <x:c r="AZ86" s="66"/>
+      <x:c r="BF86" s="66"/>
+      <x:c r="BG86" s="66"/>
     </x:row>
     <x:row r="87" ht="15" hidden="0">
       <x:c r="A87" s="18"/>
@@ -3854,6 +5162,15 @@
       <x:c r="Y87" s="49"/>
       <x:c r="Z87" s="49"/>
       <x:c r="AA87" s="49"/>
+      <x:c r="AI87" s="66"/>
+      <x:c r="AK87" s="66"/>
+      <x:c r="AM87" s="66"/>
+      <x:c r="AO87" s="66"/>
+      <x:c r="AQ87" s="66"/>
+      <x:c r="AS87" s="66"/>
+      <x:c r="AZ87" s="66"/>
+      <x:c r="BF87" s="66"/>
+      <x:c r="BG87" s="66"/>
     </x:row>
     <x:row r="88" ht="15" hidden="0">
       <x:c r="A88" s="18"/>
@@ -3885,6 +5202,15 @@
       <x:c r="Y88" s="49"/>
       <x:c r="Z88" s="49"/>
       <x:c r="AA88" s="49"/>
+      <x:c r="AI88" s="66"/>
+      <x:c r="AK88" s="66"/>
+      <x:c r="AM88" s="66"/>
+      <x:c r="AO88" s="66"/>
+      <x:c r="AQ88" s="66"/>
+      <x:c r="AS88" s="66"/>
+      <x:c r="AZ88" s="66"/>
+      <x:c r="BF88" s="66"/>
+      <x:c r="BG88" s="66"/>
     </x:row>
     <x:row r="89" ht="15" hidden="0">
       <x:c r="A89" s="18"/>
@@ -3916,6 +5242,15 @@
       <x:c r="Y89" s="49"/>
       <x:c r="Z89" s="49"/>
       <x:c r="AA89" s="49"/>
+      <x:c r="AI89" s="66"/>
+      <x:c r="AK89" s="66"/>
+      <x:c r="AM89" s="66"/>
+      <x:c r="AO89" s="66"/>
+      <x:c r="AQ89" s="66"/>
+      <x:c r="AS89" s="66"/>
+      <x:c r="AZ89" s="66"/>
+      <x:c r="BF89" s="66"/>
+      <x:c r="BG89" s="66"/>
     </x:row>
     <x:row r="90" ht="15" hidden="0">
       <x:c r="A90" s="18"/>
@@ -3947,6 +5282,15 @@
       <x:c r="Y90" s="49"/>
       <x:c r="Z90" s="49"/>
       <x:c r="AA90" s="49"/>
+      <x:c r="AI90" s="66"/>
+      <x:c r="AK90" s="66"/>
+      <x:c r="AM90" s="66"/>
+      <x:c r="AO90" s="66"/>
+      <x:c r="AQ90" s="66"/>
+      <x:c r="AS90" s="66"/>
+      <x:c r="AZ90" s="66"/>
+      <x:c r="BF90" s="66"/>
+      <x:c r="BG90" s="66"/>
     </x:row>
     <x:row r="91" ht="15" hidden="0">
       <x:c r="A91" s="18"/>
@@ -3978,6 +5322,15 @@
       <x:c r="Y91" s="49"/>
       <x:c r="Z91" s="49"/>
       <x:c r="AA91" s="49"/>
+      <x:c r="AI91" s="66"/>
+      <x:c r="AK91" s="66"/>
+      <x:c r="AM91" s="66"/>
+      <x:c r="AO91" s="66"/>
+      <x:c r="AQ91" s="66"/>
+      <x:c r="AS91" s="66"/>
+      <x:c r="AZ91" s="66"/>
+      <x:c r="BF91" s="66"/>
+      <x:c r="BG91" s="66"/>
     </x:row>
     <x:row r="92" ht="15" hidden="0">
       <x:c r="A92" s="18"/>
@@ -4009,6 +5362,15 @@
       <x:c r="Y92" s="49"/>
       <x:c r="Z92" s="49"/>
       <x:c r="AA92" s="49"/>
+      <x:c r="AI92" s="66"/>
+      <x:c r="AK92" s="66"/>
+      <x:c r="AM92" s="66"/>
+      <x:c r="AO92" s="66"/>
+      <x:c r="AQ92" s="66"/>
+      <x:c r="AS92" s="66"/>
+      <x:c r="AZ92" s="66"/>
+      <x:c r="BF92" s="66"/>
+      <x:c r="BG92" s="66"/>
     </x:row>
     <x:row r="93" ht="15" hidden="0">
       <x:c r="A93" s="18"/>
@@ -4040,6 +5402,15 @@
       <x:c r="Y93" s="49"/>
       <x:c r="Z93" s="49"/>
       <x:c r="AA93" s="49"/>
+      <x:c r="AI93" s="66"/>
+      <x:c r="AK93" s="66"/>
+      <x:c r="AM93" s="66"/>
+      <x:c r="AO93" s="66"/>
+      <x:c r="AQ93" s="66"/>
+      <x:c r="AS93" s="66"/>
+      <x:c r="AZ93" s="66"/>
+      <x:c r="BF93" s="66"/>
+      <x:c r="BG93" s="66"/>
     </x:row>
     <x:row r="94" ht="15" hidden="0">
       <x:c r="A94" s="18"/>
@@ -4071,6 +5442,15 @@
       <x:c r="Y94" s="49"/>
       <x:c r="Z94" s="49"/>
       <x:c r="AA94" s="49"/>
+      <x:c r="AI94" s="66"/>
+      <x:c r="AK94" s="66"/>
+      <x:c r="AM94" s="66"/>
+      <x:c r="AO94" s="66"/>
+      <x:c r="AQ94" s="66"/>
+      <x:c r="AS94" s="66"/>
+      <x:c r="AZ94" s="66"/>
+      <x:c r="BF94" s="66"/>
+      <x:c r="BG94" s="66"/>
     </x:row>
     <x:row r="95" ht="15" hidden="0">
       <x:c r="A95" s="18"/>
@@ -4102,6 +5482,15 @@
       <x:c r="Y95" s="49"/>
       <x:c r="Z95" s="49"/>
       <x:c r="AA95" s="49"/>
+      <x:c r="AI95" s="66"/>
+      <x:c r="AK95" s="66"/>
+      <x:c r="AM95" s="66"/>
+      <x:c r="AO95" s="66"/>
+      <x:c r="AQ95" s="66"/>
+      <x:c r="AS95" s="66"/>
+      <x:c r="AZ95" s="66"/>
+      <x:c r="BF95" s="66"/>
+      <x:c r="BG95" s="66"/>
     </x:row>
     <x:row r="96" ht="15" hidden="0">
       <x:c r="A96" s="18"/>
@@ -4133,6 +5522,15 @@
       <x:c r="Y96" s="49"/>
       <x:c r="Z96" s="49"/>
       <x:c r="AA96" s="49"/>
+      <x:c r="AI96" s="66"/>
+      <x:c r="AK96" s="66"/>
+      <x:c r="AM96" s="66"/>
+      <x:c r="AO96" s="66"/>
+      <x:c r="AQ96" s="66"/>
+      <x:c r="AS96" s="66"/>
+      <x:c r="AZ96" s="66"/>
+      <x:c r="BF96" s="66"/>
+      <x:c r="BG96" s="66"/>
     </x:row>
     <x:row r="97" ht="15" hidden="0">
       <x:c r="A97" s="18"/>
@@ -4164,6 +5562,15 @@
       <x:c r="Y97" s="49"/>
       <x:c r="Z97" s="49"/>
       <x:c r="AA97" s="49"/>
+      <x:c r="AI97" s="66"/>
+      <x:c r="AK97" s="66"/>
+      <x:c r="AM97" s="66"/>
+      <x:c r="AO97" s="66"/>
+      <x:c r="AQ97" s="66"/>
+      <x:c r="AS97" s="66"/>
+      <x:c r="AZ97" s="66"/>
+      <x:c r="BF97" s="66"/>
+      <x:c r="BG97" s="66"/>
     </x:row>
     <x:row r="98" ht="15" hidden="0">
       <x:c r="A98" s="18"/>
@@ -4195,6 +5602,15 @@
       <x:c r="Y98" s="49"/>
       <x:c r="Z98" s="49"/>
       <x:c r="AA98" s="49"/>
+      <x:c r="AI98" s="66"/>
+      <x:c r="AK98" s="66"/>
+      <x:c r="AM98" s="66"/>
+      <x:c r="AO98" s="66"/>
+      <x:c r="AQ98" s="66"/>
+      <x:c r="AS98" s="66"/>
+      <x:c r="AZ98" s="66"/>
+      <x:c r="BF98" s="66"/>
+      <x:c r="BG98" s="66"/>
     </x:row>
     <x:row r="99" ht="15" hidden="0">
       <x:c r="A99" s="18"/>
@@ -4226,6 +5642,15 @@
       <x:c r="Y99" s="49"/>
       <x:c r="Z99" s="49"/>
       <x:c r="AA99" s="49"/>
+      <x:c r="AI99" s="66"/>
+      <x:c r="AK99" s="66"/>
+      <x:c r="AM99" s="66"/>
+      <x:c r="AO99" s="66"/>
+      <x:c r="AQ99" s="66"/>
+      <x:c r="AS99" s="66"/>
+      <x:c r="AZ99" s="66"/>
+      <x:c r="BF99" s="66"/>
+      <x:c r="BG99" s="66"/>
     </x:row>
     <x:row r="100" ht="15" hidden="0">
       <x:c r="A100" s="18"/>
@@ -4257,6 +5682,15 @@
       <x:c r="Y100" s="49"/>
       <x:c r="Z100" s="49"/>
       <x:c r="AA100" s="49"/>
+      <x:c r="AI100" s="66"/>
+      <x:c r="AK100" s="66"/>
+      <x:c r="AM100" s="66"/>
+      <x:c r="AO100" s="66"/>
+      <x:c r="AQ100" s="66"/>
+      <x:c r="AS100" s="66"/>
+      <x:c r="AZ100" s="66"/>
+      <x:c r="BF100" s="66"/>
+      <x:c r="BG100" s="66"/>
     </x:row>
     <x:row r="101" ht="15" hidden="0">
       <x:c r="A101" s="18"/>
@@ -4288,6 +5722,15 @@
       <x:c r="Y101" s="49"/>
       <x:c r="Z101" s="49"/>
       <x:c r="AA101" s="49"/>
+      <x:c r="AI101" s="66"/>
+      <x:c r="AK101" s="66"/>
+      <x:c r="AM101" s="66"/>
+      <x:c r="AO101" s="66"/>
+      <x:c r="AQ101" s="66"/>
+      <x:c r="AS101" s="66"/>
+      <x:c r="AZ101" s="66"/>
+      <x:c r="BF101" s="66"/>
+      <x:c r="BG101" s="66"/>
     </x:row>
     <x:row r="102" ht="15" hidden="0">
       <x:c r="A102" s="18"/>
@@ -4319,6 +5762,15 @@
       <x:c r="Y102" s="49"/>
       <x:c r="Z102" s="49"/>
       <x:c r="AA102" s="49"/>
+      <x:c r="AI102" s="66"/>
+      <x:c r="AK102" s="66"/>
+      <x:c r="AM102" s="66"/>
+      <x:c r="AO102" s="66"/>
+      <x:c r="AQ102" s="66"/>
+      <x:c r="AS102" s="66"/>
+      <x:c r="AZ102" s="66"/>
+      <x:c r="BF102" s="66"/>
+      <x:c r="BG102" s="66"/>
     </x:row>
     <x:row r="103" ht="15" hidden="0">
       <x:c r="A103" s="18"/>
@@ -4350,6 +5802,15 @@
       <x:c r="Y103" s="49"/>
       <x:c r="Z103" s="49"/>
       <x:c r="AA103" s="49"/>
+      <x:c r="AI103" s="66"/>
+      <x:c r="AK103" s="66"/>
+      <x:c r="AM103" s="66"/>
+      <x:c r="AO103" s="66"/>
+      <x:c r="AQ103" s="66"/>
+      <x:c r="AS103" s="66"/>
+      <x:c r="AZ103" s="66"/>
+      <x:c r="BF103" s="66"/>
+      <x:c r="BG103" s="66"/>
     </x:row>
     <x:row r="104" ht="15" hidden="0">
       <x:c r="A104" s="18"/>
@@ -4381,6 +5842,15 @@
       <x:c r="Y104" s="49"/>
       <x:c r="Z104" s="49"/>
       <x:c r="AA104" s="49"/>
+      <x:c r="AI104" s="66"/>
+      <x:c r="AK104" s="66"/>
+      <x:c r="AM104" s="66"/>
+      <x:c r="AO104" s="66"/>
+      <x:c r="AQ104" s="66"/>
+      <x:c r="AS104" s="66"/>
+      <x:c r="AZ104" s="66"/>
+      <x:c r="BF104" s="66"/>
+      <x:c r="BG104" s="66"/>
     </x:row>
     <x:row r="105" ht="15" hidden="0">
       <x:c r="A105" s="18"/>
@@ -4412,6 +5882,15 @@
       <x:c r="Y105" s="49"/>
       <x:c r="Z105" s="49"/>
       <x:c r="AA105" s="49"/>
+      <x:c r="AI105" s="66"/>
+      <x:c r="AK105" s="66"/>
+      <x:c r="AM105" s="66"/>
+      <x:c r="AO105" s="66"/>
+      <x:c r="AQ105" s="66"/>
+      <x:c r="AS105" s="66"/>
+      <x:c r="AZ105" s="66"/>
+      <x:c r="BF105" s="66"/>
+      <x:c r="BG105" s="66"/>
     </x:row>
     <x:row r="106" ht="15" hidden="0">
       <x:c r="A106" s="18"/>
@@ -4443,6 +5922,15 @@
       <x:c r="Y106" s="49"/>
       <x:c r="Z106" s="49"/>
       <x:c r="AA106" s="49"/>
+      <x:c r="AI106" s="66"/>
+      <x:c r="AK106" s="66"/>
+      <x:c r="AM106" s="66"/>
+      <x:c r="AO106" s="66"/>
+      <x:c r="AQ106" s="66"/>
+      <x:c r="AS106" s="66"/>
+      <x:c r="AZ106" s="66"/>
+      <x:c r="BF106" s="66"/>
+      <x:c r="BG106" s="66"/>
     </x:row>
     <x:row r="107" ht="15" hidden="0">
       <x:c r="A107" s="18"/>
@@ -4474,6 +5962,15 @@
       <x:c r="Y107" s="49"/>
       <x:c r="Z107" s="49"/>
       <x:c r="AA107" s="49"/>
+      <x:c r="AI107" s="66"/>
+      <x:c r="AK107" s="66"/>
+      <x:c r="AM107" s="66"/>
+      <x:c r="AO107" s="66"/>
+      <x:c r="AQ107" s="66"/>
+      <x:c r="AS107" s="66"/>
+      <x:c r="AZ107" s="66"/>
+      <x:c r="BF107" s="66"/>
+      <x:c r="BG107" s="66"/>
     </x:row>
     <x:row r="108" ht="15" hidden="0">
       <x:c r="A108" s="18"/>
@@ -4505,6 +6002,15 @@
       <x:c r="Y108" s="49"/>
       <x:c r="Z108" s="49"/>
       <x:c r="AA108" s="49"/>
+      <x:c r="AI108" s="66"/>
+      <x:c r="AK108" s="66"/>
+      <x:c r="AM108" s="66"/>
+      <x:c r="AO108" s="66"/>
+      <x:c r="AQ108" s="66"/>
+      <x:c r="AS108" s="66"/>
+      <x:c r="AZ108" s="66"/>
+      <x:c r="BF108" s="66"/>
+      <x:c r="BG108" s="66"/>
     </x:row>
     <x:row r="109" ht="15" hidden="0">
       <x:c r="A109" s="18"/>
@@ -4536,6 +6042,15 @@
       <x:c r="Y109" s="49"/>
       <x:c r="Z109" s="49"/>
       <x:c r="AA109" s="49"/>
+      <x:c r="AI109" s="66"/>
+      <x:c r="AK109" s="66"/>
+      <x:c r="AM109" s="66"/>
+      <x:c r="AO109" s="66"/>
+      <x:c r="AQ109" s="66"/>
+      <x:c r="AS109" s="66"/>
+      <x:c r="AZ109" s="66"/>
+      <x:c r="BF109" s="66"/>
+      <x:c r="BG109" s="66"/>
     </x:row>
     <x:row r="110" ht="15" hidden="0">
       <x:c r="A110" s="18"/>
@@ -4567,6 +6082,15 @@
       <x:c r="Y110" s="49"/>
       <x:c r="Z110" s="49"/>
       <x:c r="AA110" s="49"/>
+      <x:c r="AI110" s="66"/>
+      <x:c r="AK110" s="66"/>
+      <x:c r="AM110" s="66"/>
+      <x:c r="AO110" s="66"/>
+      <x:c r="AQ110" s="66"/>
+      <x:c r="AS110" s="66"/>
+      <x:c r="AZ110" s="66"/>
+      <x:c r="BF110" s="66"/>
+      <x:c r="BG110" s="66"/>
     </x:row>
     <x:row r="111" ht="15" hidden="0">
       <x:c r="A111" s="18"/>
@@ -4598,6 +6122,15 @@
       <x:c r="Y111" s="49"/>
       <x:c r="Z111" s="49"/>
       <x:c r="AA111" s="49"/>
+      <x:c r="AI111" s="66"/>
+      <x:c r="AK111" s="66"/>
+      <x:c r="AM111" s="66"/>
+      <x:c r="AO111" s="66"/>
+      <x:c r="AQ111" s="66"/>
+      <x:c r="AS111" s="66"/>
+      <x:c r="AZ111" s="66"/>
+      <x:c r="BF111" s="66"/>
+      <x:c r="BG111" s="66"/>
     </x:row>
     <x:row r="112" ht="15" hidden="0">
       <x:c r="A112" s="18"/>
@@ -4629,6 +6162,15 @@
       <x:c r="Y112" s="49"/>
       <x:c r="Z112" s="49"/>
       <x:c r="AA112" s="49"/>
+      <x:c r="AI112" s="66"/>
+      <x:c r="AK112" s="66"/>
+      <x:c r="AM112" s="66"/>
+      <x:c r="AO112" s="66"/>
+      <x:c r="AQ112" s="66"/>
+      <x:c r="AS112" s="66"/>
+      <x:c r="AZ112" s="66"/>
+      <x:c r="BF112" s="66"/>
+      <x:c r="BG112" s="66"/>
     </x:row>
     <x:row r="113" ht="15" hidden="0">
       <x:c r="A113" s="18"/>
@@ -4660,6 +6202,15 @@
       <x:c r="Y113" s="49"/>
       <x:c r="Z113" s="49"/>
       <x:c r="AA113" s="49"/>
+      <x:c r="AI113" s="66"/>
+      <x:c r="AK113" s="66"/>
+      <x:c r="AM113" s="66"/>
+      <x:c r="AO113" s="66"/>
+      <x:c r="AQ113" s="66"/>
+      <x:c r="AS113" s="66"/>
+      <x:c r="AZ113" s="66"/>
+      <x:c r="BF113" s="66"/>
+      <x:c r="BG113" s="66"/>
     </x:row>
     <x:row r="114" ht="15" hidden="0">
       <x:c r="A114" s="18"/>
@@ -4691,6 +6242,15 @@
       <x:c r="Y114" s="49"/>
       <x:c r="Z114" s="49"/>
       <x:c r="AA114" s="49"/>
+      <x:c r="AI114" s="66"/>
+      <x:c r="AK114" s="66"/>
+      <x:c r="AM114" s="66"/>
+      <x:c r="AO114" s="66"/>
+      <x:c r="AQ114" s="66"/>
+      <x:c r="AS114" s="66"/>
+      <x:c r="AZ114" s="66"/>
+      <x:c r="BF114" s="66"/>
+      <x:c r="BG114" s="66"/>
     </x:row>
     <x:row r="115" ht="15" hidden="0">
       <x:c r="A115" s="18"/>
@@ -4722,6 +6282,15 @@
       <x:c r="Y115" s="49"/>
       <x:c r="Z115" s="49"/>
       <x:c r="AA115" s="49"/>
+      <x:c r="AI115" s="66"/>
+      <x:c r="AK115" s="66"/>
+      <x:c r="AM115" s="66"/>
+      <x:c r="AO115" s="66"/>
+      <x:c r="AQ115" s="66"/>
+      <x:c r="AS115" s="66"/>
+      <x:c r="AZ115" s="66"/>
+      <x:c r="BF115" s="66"/>
+      <x:c r="BG115" s="66"/>
     </x:row>
     <x:row r="116" ht="15" hidden="0">
       <x:c r="A116" s="18"/>
@@ -4753,6 +6322,15 @@
       <x:c r="Y116" s="49"/>
       <x:c r="Z116" s="49"/>
       <x:c r="AA116" s="49"/>
+      <x:c r="AI116" s="66"/>
+      <x:c r="AK116" s="66"/>
+      <x:c r="AM116" s="66"/>
+      <x:c r="AO116" s="66"/>
+      <x:c r="AQ116" s="66"/>
+      <x:c r="AS116" s="66"/>
+      <x:c r="AZ116" s="66"/>
+      <x:c r="BF116" s="66"/>
+      <x:c r="BG116" s="66"/>
     </x:row>
     <x:row r="117" ht="15" hidden="0">
       <x:c r="A117" s="18"/>
@@ -4784,6 +6362,15 @@
       <x:c r="Y117" s="49"/>
       <x:c r="Z117" s="49"/>
       <x:c r="AA117" s="49"/>
+      <x:c r="AI117" s="66"/>
+      <x:c r="AK117" s="66"/>
+      <x:c r="AM117" s="66"/>
+      <x:c r="AO117" s="66"/>
+      <x:c r="AQ117" s="66"/>
+      <x:c r="AS117" s="66"/>
+      <x:c r="AZ117" s="66"/>
+      <x:c r="BF117" s="66"/>
+      <x:c r="BG117" s="66"/>
     </x:row>
     <x:row r="118" ht="15" hidden="0">
       <x:c r="A118" s="18"/>
@@ -4815,6 +6402,15 @@
       <x:c r="Y118" s="49"/>
       <x:c r="Z118" s="49"/>
       <x:c r="AA118" s="49"/>
+      <x:c r="AI118" s="66"/>
+      <x:c r="AK118" s="66"/>
+      <x:c r="AM118" s="66"/>
+      <x:c r="AO118" s="66"/>
+      <x:c r="AQ118" s="66"/>
+      <x:c r="AS118" s="66"/>
+      <x:c r="AZ118" s="66"/>
+      <x:c r="BF118" s="66"/>
+      <x:c r="BG118" s="66"/>
     </x:row>
     <x:row r="119" ht="15" hidden="0">
       <x:c r="A119" s="18"/>
@@ -4846,6 +6442,15 @@
       <x:c r="Y119" s="49"/>
       <x:c r="Z119" s="49"/>
       <x:c r="AA119" s="49"/>
+      <x:c r="AI119" s="66"/>
+      <x:c r="AK119" s="66"/>
+      <x:c r="AM119" s="66"/>
+      <x:c r="AO119" s="66"/>
+      <x:c r="AQ119" s="66"/>
+      <x:c r="AS119" s="66"/>
+      <x:c r="AZ119" s="66"/>
+      <x:c r="BF119" s="66"/>
+      <x:c r="BG119" s="66"/>
     </x:row>
     <x:row r="120" ht="15" hidden="0">
       <x:c r="A120" s="18"/>
@@ -4877,6 +6482,15 @@
       <x:c r="Y120" s="49"/>
       <x:c r="Z120" s="49"/>
       <x:c r="AA120" s="49"/>
+      <x:c r="AI120" s="66"/>
+      <x:c r="AK120" s="66"/>
+      <x:c r="AM120" s="66"/>
+      <x:c r="AO120" s="66"/>
+      <x:c r="AQ120" s="66"/>
+      <x:c r="AS120" s="66"/>
+      <x:c r="AZ120" s="66"/>
+      <x:c r="BF120" s="66"/>
+      <x:c r="BG120" s="66"/>
     </x:row>
     <x:row r="121" ht="15" hidden="0">
       <x:c r="A121" s="18"/>
@@ -4908,6 +6522,15 @@
       <x:c r="Y121" s="49"/>
       <x:c r="Z121" s="49"/>
       <x:c r="AA121" s="49"/>
+      <x:c r="AI121" s="66"/>
+      <x:c r="AK121" s="66"/>
+      <x:c r="AM121" s="66"/>
+      <x:c r="AO121" s="66"/>
+      <x:c r="AQ121" s="66"/>
+      <x:c r="AS121" s="66"/>
+      <x:c r="AZ121" s="66"/>
+      <x:c r="BF121" s="66"/>
+      <x:c r="BG121" s="66"/>
     </x:row>
     <x:row r="122" ht="15" hidden="0">
       <x:c r="A122" s="18"/>
@@ -4939,6 +6562,15 @@
       <x:c r="Y122" s="49"/>
       <x:c r="Z122" s="49"/>
       <x:c r="AA122" s="49"/>
+      <x:c r="AI122" s="66"/>
+      <x:c r="AK122" s="66"/>
+      <x:c r="AM122" s="66"/>
+      <x:c r="AO122" s="66"/>
+      <x:c r="AQ122" s="66"/>
+      <x:c r="AS122" s="66"/>
+      <x:c r="AZ122" s="66"/>
+      <x:c r="BF122" s="66"/>
+      <x:c r="BG122" s="66"/>
     </x:row>
     <x:row r="123" ht="15" hidden="0">
       <x:c r="A123" s="18"/>
@@ -4970,6 +6602,15 @@
       <x:c r="Y123" s="49"/>
       <x:c r="Z123" s="49"/>
       <x:c r="AA123" s="49"/>
+      <x:c r="AI123" s="66"/>
+      <x:c r="AK123" s="66"/>
+      <x:c r="AM123" s="66"/>
+      <x:c r="AO123" s="66"/>
+      <x:c r="AQ123" s="66"/>
+      <x:c r="AS123" s="66"/>
+      <x:c r="AZ123" s="66"/>
+      <x:c r="BF123" s="66"/>
+      <x:c r="BG123" s="66"/>
     </x:row>
     <x:row r="124" ht="15" hidden="0">
       <x:c r="A124" s="18"/>
@@ -5001,6 +6642,15 @@
       <x:c r="Y124" s="49"/>
       <x:c r="Z124" s="49"/>
       <x:c r="AA124" s="49"/>
+      <x:c r="AI124" s="66"/>
+      <x:c r="AK124" s="66"/>
+      <x:c r="AM124" s="66"/>
+      <x:c r="AO124" s="66"/>
+      <x:c r="AQ124" s="66"/>
+      <x:c r="AS124" s="66"/>
+      <x:c r="AZ124" s="66"/>
+      <x:c r="BF124" s="66"/>
+      <x:c r="BG124" s="66"/>
     </x:row>
     <x:row r="125" ht="15" hidden="0">
       <x:c r="A125" s="18"/>
@@ -5032,6 +6682,15 @@
       <x:c r="Y125" s="49"/>
       <x:c r="Z125" s="49"/>
       <x:c r="AA125" s="49"/>
+      <x:c r="AI125" s="66"/>
+      <x:c r="AK125" s="66"/>
+      <x:c r="AM125" s="66"/>
+      <x:c r="AO125" s="66"/>
+      <x:c r="AQ125" s="66"/>
+      <x:c r="AS125" s="66"/>
+      <x:c r="AZ125" s="66"/>
+      <x:c r="BF125" s="66"/>
+      <x:c r="BG125" s="66"/>
     </x:row>
     <x:row r="126" ht="15" hidden="0">
       <x:c r="A126" s="18"/>
@@ -5063,6 +6722,15 @@
       <x:c r="Y126" s="49"/>
       <x:c r="Z126" s="49"/>
       <x:c r="AA126" s="49"/>
+      <x:c r="AI126" s="66"/>
+      <x:c r="AK126" s="66"/>
+      <x:c r="AM126" s="66"/>
+      <x:c r="AO126" s="66"/>
+      <x:c r="AQ126" s="66"/>
+      <x:c r="AS126" s="66"/>
+      <x:c r="AZ126" s="66"/>
+      <x:c r="BF126" s="66"/>
+      <x:c r="BG126" s="66"/>
     </x:row>
     <x:row r="127" ht="15" hidden="0">
       <x:c r="A127" s="18"/>
@@ -5094,6 +6762,15 @@
       <x:c r="Y127" s="49"/>
       <x:c r="Z127" s="49"/>
       <x:c r="AA127" s="49"/>
+      <x:c r="AI127" s="66"/>
+      <x:c r="AK127" s="66"/>
+      <x:c r="AM127" s="66"/>
+      <x:c r="AO127" s="66"/>
+      <x:c r="AQ127" s="66"/>
+      <x:c r="AS127" s="66"/>
+      <x:c r="AZ127" s="66"/>
+      <x:c r="BF127" s="66"/>
+      <x:c r="BG127" s="66"/>
     </x:row>
     <x:row r="128" ht="15" hidden="0">
       <x:c r="A128" s="18"/>
@@ -5125,6 +6802,15 @@
       <x:c r="Y128" s="49"/>
       <x:c r="Z128" s="49"/>
       <x:c r="AA128" s="49"/>
+      <x:c r="AI128" s="66"/>
+      <x:c r="AK128" s="66"/>
+      <x:c r="AM128" s="66"/>
+      <x:c r="AO128" s="66"/>
+      <x:c r="AQ128" s="66"/>
+      <x:c r="AS128" s="66"/>
+      <x:c r="AZ128" s="66"/>
+      <x:c r="BF128" s="66"/>
+      <x:c r="BG128" s="66"/>
     </x:row>
     <x:row r="129" ht="15" hidden="0">
       <x:c r="A129" s="18"/>
@@ -5156,6 +6842,15 @@
       <x:c r="Y129" s="49"/>
       <x:c r="Z129" s="49"/>
       <x:c r="AA129" s="49"/>
+      <x:c r="AI129" s="66"/>
+      <x:c r="AK129" s="66"/>
+      <x:c r="AM129" s="66"/>
+      <x:c r="AO129" s="66"/>
+      <x:c r="AQ129" s="66"/>
+      <x:c r="AS129" s="66"/>
+      <x:c r="AZ129" s="66"/>
+      <x:c r="BF129" s="66"/>
+      <x:c r="BG129" s="66"/>
     </x:row>
     <x:row r="130" ht="15" hidden="0">
       <x:c r="A130" s="18"/>
@@ -5187,6 +6882,15 @@
       <x:c r="Y130" s="49"/>
       <x:c r="Z130" s="49"/>
       <x:c r="AA130" s="49"/>
+      <x:c r="AI130" s="66"/>
+      <x:c r="AK130" s="66"/>
+      <x:c r="AM130" s="66"/>
+      <x:c r="AO130" s="66"/>
+      <x:c r="AQ130" s="66"/>
+      <x:c r="AS130" s="66"/>
+      <x:c r="AZ130" s="66"/>
+      <x:c r="BF130" s="66"/>
+      <x:c r="BG130" s="66"/>
     </x:row>
     <x:row r="131" ht="15" hidden="0">
       <x:c r="A131" s="18"/>
@@ -5218,6 +6922,15 @@
       <x:c r="Y131" s="49"/>
       <x:c r="Z131" s="49"/>
       <x:c r="AA131" s="49"/>
+      <x:c r="AI131" s="66"/>
+      <x:c r="AK131" s="66"/>
+      <x:c r="AM131" s="66"/>
+      <x:c r="AO131" s="66"/>
+      <x:c r="AQ131" s="66"/>
+      <x:c r="AS131" s="66"/>
+      <x:c r="AZ131" s="66"/>
+      <x:c r="BF131" s="66"/>
+      <x:c r="BG131" s="66"/>
     </x:row>
     <x:row r="132" ht="15" hidden="0">
       <x:c r="A132" s="18"/>
@@ -5249,6 +6962,15 @@
       <x:c r="Y132" s="49"/>
       <x:c r="Z132" s="49"/>
       <x:c r="AA132" s="49"/>
+      <x:c r="AI132" s="66"/>
+      <x:c r="AK132" s="66"/>
+      <x:c r="AM132" s="66"/>
+      <x:c r="AO132" s="66"/>
+      <x:c r="AQ132" s="66"/>
+      <x:c r="AS132" s="66"/>
+      <x:c r="AZ132" s="66"/>
+      <x:c r="BF132" s="66"/>
+      <x:c r="BG132" s="66"/>
     </x:row>
     <x:row r="133" ht="15" hidden="0">
       <x:c r="A133" s="18"/>
@@ -5280,6 +7002,15 @@
       <x:c r="Y133" s="49"/>
       <x:c r="Z133" s="49"/>
       <x:c r="AA133" s="49"/>
+      <x:c r="AI133" s="66"/>
+      <x:c r="AK133" s="66"/>
+      <x:c r="AM133" s="66"/>
+      <x:c r="AO133" s="66"/>
+      <x:c r="AQ133" s="66"/>
+      <x:c r="AS133" s="66"/>
+      <x:c r="AZ133" s="66"/>
+      <x:c r="BF133" s="66"/>
+      <x:c r="BG133" s="66"/>
     </x:row>
     <x:row r="134" ht="15" hidden="0">
       <x:c r="A134" s="18"/>
@@ -5311,6 +7042,15 @@
       <x:c r="Y134" s="49"/>
       <x:c r="Z134" s="49"/>
       <x:c r="AA134" s="49"/>
+      <x:c r="AI134" s="66"/>
+      <x:c r="AK134" s="66"/>
+      <x:c r="AM134" s="66"/>
+      <x:c r="AO134" s="66"/>
+      <x:c r="AQ134" s="66"/>
+      <x:c r="AS134" s="66"/>
+      <x:c r="AZ134" s="66"/>
+      <x:c r="BF134" s="66"/>
+      <x:c r="BG134" s="66"/>
     </x:row>
     <x:row r="135" ht="15" hidden="0">
       <x:c r="A135" s="18"/>
@@ -5342,6 +7082,15 @@
       <x:c r="Y135" s="49"/>
       <x:c r="Z135" s="49"/>
       <x:c r="AA135" s="49"/>
+      <x:c r="AI135" s="66"/>
+      <x:c r="AK135" s="66"/>
+      <x:c r="AM135" s="66"/>
+      <x:c r="AO135" s="66"/>
+      <x:c r="AQ135" s="66"/>
+      <x:c r="AS135" s="66"/>
+      <x:c r="AZ135" s="66"/>
+      <x:c r="BF135" s="66"/>
+      <x:c r="BG135" s="66"/>
     </x:row>
     <x:row r="136" ht="15" hidden="0">
       <x:c r="A136" s="18"/>
@@ -5373,6 +7122,15 @@
       <x:c r="Y136" s="49"/>
       <x:c r="Z136" s="49"/>
       <x:c r="AA136" s="49"/>
+      <x:c r="AI136" s="66"/>
+      <x:c r="AK136" s="66"/>
+      <x:c r="AM136" s="66"/>
+      <x:c r="AO136" s="66"/>
+      <x:c r="AQ136" s="66"/>
+      <x:c r="AS136" s="66"/>
+      <x:c r="AZ136" s="66"/>
+      <x:c r="BF136" s="66"/>
+      <x:c r="BG136" s="66"/>
     </x:row>
     <x:row r="137" ht="15" hidden="0">
       <x:c r="A137" s="18"/>
@@ -5404,6 +7162,15 @@
       <x:c r="Y137" s="49"/>
       <x:c r="Z137" s="49"/>
       <x:c r="AA137" s="49"/>
+      <x:c r="AI137" s="66"/>
+      <x:c r="AK137" s="66"/>
+      <x:c r="AM137" s="66"/>
+      <x:c r="AO137" s="66"/>
+      <x:c r="AQ137" s="66"/>
+      <x:c r="AS137" s="66"/>
+      <x:c r="AZ137" s="66"/>
+      <x:c r="BF137" s="66"/>
+      <x:c r="BG137" s="66"/>
     </x:row>
     <x:row r="138" ht="15" hidden="0">
       <x:c r="A138" s="18"/>
@@ -5435,6 +7202,15 @@
       <x:c r="Y138" s="49"/>
       <x:c r="Z138" s="49"/>
       <x:c r="AA138" s="49"/>
+      <x:c r="AI138" s="66"/>
+      <x:c r="AK138" s="66"/>
+      <x:c r="AM138" s="66"/>
+      <x:c r="AO138" s="66"/>
+      <x:c r="AQ138" s="66"/>
+      <x:c r="AS138" s="66"/>
+      <x:c r="AZ138" s="66"/>
+      <x:c r="BF138" s="66"/>
+      <x:c r="BG138" s="66"/>
     </x:row>
     <x:row r="139" ht="15" hidden="0">
       <x:c r="A139" s="18"/>
@@ -5466,6 +7242,15 @@
       <x:c r="Y139" s="49"/>
       <x:c r="Z139" s="49"/>
       <x:c r="AA139" s="49"/>
+      <x:c r="AI139" s="66"/>
+      <x:c r="AK139" s="66"/>
+      <x:c r="AM139" s="66"/>
+      <x:c r="AO139" s="66"/>
+      <x:c r="AQ139" s="66"/>
+      <x:c r="AS139" s="66"/>
+      <x:c r="AZ139" s="66"/>
+      <x:c r="BF139" s="66"/>
+      <x:c r="BG139" s="66"/>
     </x:row>
     <x:row r="140" ht="15" hidden="0">
       <x:c r="A140" s="18"/>
@@ -5497,6 +7282,15 @@
       <x:c r="Y140" s="49"/>
       <x:c r="Z140" s="49"/>
       <x:c r="AA140" s="49"/>
+      <x:c r="AI140" s="66"/>
+      <x:c r="AK140" s="66"/>
+      <x:c r="AM140" s="66"/>
+      <x:c r="AO140" s="66"/>
+      <x:c r="AQ140" s="66"/>
+      <x:c r="AS140" s="66"/>
+      <x:c r="AZ140" s="66"/>
+      <x:c r="BF140" s="66"/>
+      <x:c r="BG140" s="66"/>
     </x:row>
     <x:row r="141" ht="15" hidden="0">
       <x:c r="A141" s="18"/>
@@ -5528,6 +7322,15 @@
       <x:c r="Y141" s="49"/>
       <x:c r="Z141" s="49"/>
       <x:c r="AA141" s="49"/>
+      <x:c r="AI141" s="66"/>
+      <x:c r="AK141" s="66"/>
+      <x:c r="AM141" s="66"/>
+      <x:c r="AO141" s="66"/>
+      <x:c r="AQ141" s="66"/>
+      <x:c r="AS141" s="66"/>
+      <x:c r="AZ141" s="66"/>
+      <x:c r="BF141" s="66"/>
+      <x:c r="BG141" s="66"/>
     </x:row>
     <x:row r="142" ht="15" hidden="0">
       <x:c r="A142" s="18"/>
@@ -5559,6 +7362,15 @@
       <x:c r="Y142" s="49"/>
       <x:c r="Z142" s="49"/>
       <x:c r="AA142" s="49"/>
+      <x:c r="AI142" s="66"/>
+      <x:c r="AK142" s="66"/>
+      <x:c r="AM142" s="66"/>
+      <x:c r="AO142" s="66"/>
+      <x:c r="AQ142" s="66"/>
+      <x:c r="AS142" s="66"/>
+      <x:c r="AZ142" s="66"/>
+      <x:c r="BF142" s="66"/>
+      <x:c r="BG142" s="66"/>
     </x:row>
     <x:row r="143" ht="15" hidden="0">
       <x:c r="A143" s="18"/>
@@ -5590,6 +7402,15 @@
       <x:c r="Y143" s="49"/>
       <x:c r="Z143" s="49"/>
       <x:c r="AA143" s="49"/>
+      <x:c r="AI143" s="66"/>
+      <x:c r="AK143" s="66"/>
+      <x:c r="AM143" s="66"/>
+      <x:c r="AO143" s="66"/>
+      <x:c r="AQ143" s="66"/>
+      <x:c r="AS143" s="66"/>
+      <x:c r="AZ143" s="66"/>
+      <x:c r="BF143" s="66"/>
+      <x:c r="BG143" s="66"/>
     </x:row>
     <x:row r="144" ht="15" hidden="0">
       <x:c r="A144" s="18"/>
@@ -5621,6 +7442,15 @@
       <x:c r="Y144" s="49"/>
       <x:c r="Z144" s="49"/>
       <x:c r="AA144" s="49"/>
+      <x:c r="AI144" s="66"/>
+      <x:c r="AK144" s="66"/>
+      <x:c r="AM144" s="66"/>
+      <x:c r="AO144" s="66"/>
+      <x:c r="AQ144" s="66"/>
+      <x:c r="AS144" s="66"/>
+      <x:c r="AZ144" s="66"/>
+      <x:c r="BF144" s="66"/>
+      <x:c r="BG144" s="66"/>
     </x:row>
     <x:row r="145" ht="15" hidden="0">
       <x:c r="A145" s="18"/>
@@ -5652,6 +7482,15 @@
       <x:c r="Y145" s="49"/>
       <x:c r="Z145" s="49"/>
       <x:c r="AA145" s="49"/>
+      <x:c r="AI145" s="66"/>
+      <x:c r="AK145" s="66"/>
+      <x:c r="AM145" s="66"/>
+      <x:c r="AO145" s="66"/>
+      <x:c r="AQ145" s="66"/>
+      <x:c r="AS145" s="66"/>
+      <x:c r="AZ145" s="66"/>
+      <x:c r="BF145" s="66"/>
+      <x:c r="BG145" s="66"/>
     </x:row>
     <x:row r="146" ht="15" hidden="0">
       <x:c r="A146" s="18"/>
@@ -5683,6 +7522,15 @@
       <x:c r="Y146" s="49"/>
       <x:c r="Z146" s="49"/>
       <x:c r="AA146" s="49"/>
+      <x:c r="AI146" s="66"/>
+      <x:c r="AK146" s="66"/>
+      <x:c r="AM146" s="66"/>
+      <x:c r="AO146" s="66"/>
+      <x:c r="AQ146" s="66"/>
+      <x:c r="AS146" s="66"/>
+      <x:c r="AZ146" s="66"/>
+      <x:c r="BF146" s="66"/>
+      <x:c r="BG146" s="66"/>
     </x:row>
     <x:row r="147" ht="15" hidden="0">
       <x:c r="A147" s="18"/>
@@ -5714,6 +7562,15 @@
       <x:c r="Y147" s="49"/>
       <x:c r="Z147" s="49"/>
       <x:c r="AA147" s="49"/>
+      <x:c r="AI147" s="66"/>
+      <x:c r="AK147" s="66"/>
+      <x:c r="AM147" s="66"/>
+      <x:c r="AO147" s="66"/>
+      <x:c r="AQ147" s="66"/>
+      <x:c r="AS147" s="66"/>
+      <x:c r="AZ147" s="66"/>
+      <x:c r="BF147" s="66"/>
+      <x:c r="BG147" s="66"/>
     </x:row>
     <x:row r="148" ht="15" hidden="0">
       <x:c r="A148" s="18"/>
@@ -5745,6 +7602,15 @@
       <x:c r="Y148" s="49"/>
       <x:c r="Z148" s="49"/>
       <x:c r="AA148" s="49"/>
+      <x:c r="AI148" s="66"/>
+      <x:c r="AK148" s="66"/>
+      <x:c r="AM148" s="66"/>
+      <x:c r="AO148" s="66"/>
+      <x:c r="AQ148" s="66"/>
+      <x:c r="AS148" s="66"/>
+      <x:c r="AZ148" s="66"/>
+      <x:c r="BF148" s="66"/>
+      <x:c r="BG148" s="66"/>
     </x:row>
     <x:row r="149" ht="15" hidden="0">
       <x:c r="A149" s="18"/>
@@ -5776,6 +7642,15 @@
       <x:c r="Y149" s="49"/>
       <x:c r="Z149" s="49"/>
       <x:c r="AA149" s="49"/>
+      <x:c r="AI149" s="66"/>
+      <x:c r="AK149" s="66"/>
+      <x:c r="AM149" s="66"/>
+      <x:c r="AO149" s="66"/>
+      <x:c r="AQ149" s="66"/>
+      <x:c r="AS149" s="66"/>
+      <x:c r="AZ149" s="66"/>
+      <x:c r="BF149" s="66"/>
+      <x:c r="BG149" s="66"/>
     </x:row>
     <x:row r="150" ht="15" hidden="0">
       <x:c r="A150" s="18"/>
@@ -5807,6 +7682,15 @@
       <x:c r="Y150" s="49"/>
       <x:c r="Z150" s="49"/>
       <x:c r="AA150" s="49"/>
+      <x:c r="AI150" s="66"/>
+      <x:c r="AK150" s="66"/>
+      <x:c r="AM150" s="66"/>
+      <x:c r="AO150" s="66"/>
+      <x:c r="AQ150" s="66"/>
+      <x:c r="AS150" s="66"/>
+      <x:c r="AZ150" s="66"/>
+      <x:c r="BF150" s="66"/>
+      <x:c r="BG150" s="66"/>
     </x:row>
     <x:row r="151" ht="15" hidden="0">
       <x:c r="A151" s="18"/>
@@ -5838,6 +7722,15 @@
       <x:c r="Y151" s="49"/>
       <x:c r="Z151" s="49"/>
       <x:c r="AA151" s="49"/>
+      <x:c r="AI151" s="66"/>
+      <x:c r="AK151" s="66"/>
+      <x:c r="AM151" s="66"/>
+      <x:c r="AO151" s="66"/>
+      <x:c r="AQ151" s="66"/>
+      <x:c r="AS151" s="66"/>
+      <x:c r="AZ151" s="66"/>
+      <x:c r="BF151" s="66"/>
+      <x:c r="BG151" s="66"/>
     </x:row>
     <x:row r="152" ht="15" hidden="0">
       <x:c r="A152" s="18"/>
@@ -5869,6 +7762,15 @@
       <x:c r="Y152" s="49"/>
       <x:c r="Z152" s="49"/>
       <x:c r="AA152" s="49"/>
+      <x:c r="AI152" s="66"/>
+      <x:c r="AK152" s="66"/>
+      <x:c r="AM152" s="66"/>
+      <x:c r="AO152" s="66"/>
+      <x:c r="AQ152" s="66"/>
+      <x:c r="AS152" s="66"/>
+      <x:c r="AZ152" s="66"/>
+      <x:c r="BF152" s="66"/>
+      <x:c r="BG152" s="66"/>
     </x:row>
     <x:row r="153" ht="15" hidden="0">
       <x:c r="A153" s="18"/>
@@ -5900,6 +7802,15 @@
       <x:c r="Y153" s="49"/>
       <x:c r="Z153" s="49"/>
       <x:c r="AA153" s="49"/>
+      <x:c r="AI153" s="66"/>
+      <x:c r="AK153" s="66"/>
+      <x:c r="AM153" s="66"/>
+      <x:c r="AO153" s="66"/>
+      <x:c r="AQ153" s="66"/>
+      <x:c r="AS153" s="66"/>
+      <x:c r="AZ153" s="66"/>
+      <x:c r="BF153" s="66"/>
+      <x:c r="BG153" s="66"/>
     </x:row>
     <x:row r="154" ht="15" hidden="0">
       <x:c r="A154" s="18"/>
@@ -5931,6 +7842,15 @@
       <x:c r="Y154" s="49"/>
       <x:c r="Z154" s="49"/>
       <x:c r="AA154" s="49"/>
+      <x:c r="AI154" s="66"/>
+      <x:c r="AK154" s="66"/>
+      <x:c r="AM154" s="66"/>
+      <x:c r="AO154" s="66"/>
+      <x:c r="AQ154" s="66"/>
+      <x:c r="AS154" s="66"/>
+      <x:c r="AZ154" s="66"/>
+      <x:c r="BF154" s="66"/>
+      <x:c r="BG154" s="66"/>
     </x:row>
     <x:row r="155" ht="15" hidden="0">
       <x:c r="A155" s="18"/>
@@ -5962,6 +7882,15 @@
       <x:c r="Y155" s="49"/>
       <x:c r="Z155" s="49"/>
       <x:c r="AA155" s="49"/>
+      <x:c r="AI155" s="66"/>
+      <x:c r="AK155" s="66"/>
+      <x:c r="AM155" s="66"/>
+      <x:c r="AO155" s="66"/>
+      <x:c r="AQ155" s="66"/>
+      <x:c r="AS155" s="66"/>
+      <x:c r="AZ155" s="66"/>
+      <x:c r="BF155" s="66"/>
+      <x:c r="BG155" s="66"/>
     </x:row>
     <x:row r="156" ht="15" hidden="0">
       <x:c r="A156" s="18"/>
@@ -5993,6 +7922,15 @@
       <x:c r="Y156" s="49"/>
       <x:c r="Z156" s="49"/>
       <x:c r="AA156" s="49"/>
+      <x:c r="AI156" s="66"/>
+      <x:c r="AK156" s="66"/>
+      <x:c r="AM156" s="66"/>
+      <x:c r="AO156" s="66"/>
+      <x:c r="AQ156" s="66"/>
+      <x:c r="AS156" s="66"/>
+      <x:c r="AZ156" s="66"/>
+      <x:c r="BF156" s="66"/>
+      <x:c r="BG156" s="66"/>
     </x:row>
     <x:row r="157" ht="15" hidden="0">
       <x:c r="A157" s="18"/>
@@ -6024,6 +7962,15 @@
       <x:c r="Y157" s="49"/>
       <x:c r="Z157" s="49"/>
       <x:c r="AA157" s="49"/>
+      <x:c r="AI157" s="66"/>
+      <x:c r="AK157" s="66"/>
+      <x:c r="AM157" s="66"/>
+      <x:c r="AO157" s="66"/>
+      <x:c r="AQ157" s="66"/>
+      <x:c r="AS157" s="66"/>
+      <x:c r="AZ157" s="66"/>
+      <x:c r="BF157" s="66"/>
+      <x:c r="BG157" s="66"/>
     </x:row>
     <x:row r="158" ht="15" hidden="0">
       <x:c r="A158" s="18"/>
@@ -6055,6 +8002,15 @@
       <x:c r="Y158" s="49"/>
       <x:c r="Z158" s="49"/>
       <x:c r="AA158" s="49"/>
+      <x:c r="AI158" s="66"/>
+      <x:c r="AK158" s="66"/>
+      <x:c r="AM158" s="66"/>
+      <x:c r="AO158" s="66"/>
+      <x:c r="AQ158" s="66"/>
+      <x:c r="AS158" s="66"/>
+      <x:c r="AZ158" s="66"/>
+      <x:c r="BF158" s="66"/>
+      <x:c r="BG158" s="66"/>
     </x:row>
     <x:row r="159" ht="15" hidden="0">
       <x:c r="A159" s="18"/>
@@ -6086,6 +8042,15 @@
       <x:c r="Y159" s="49"/>
       <x:c r="Z159" s="49"/>
       <x:c r="AA159" s="49"/>
+      <x:c r="AI159" s="66"/>
+      <x:c r="AK159" s="66"/>
+      <x:c r="AM159" s="66"/>
+      <x:c r="AO159" s="66"/>
+      <x:c r="AQ159" s="66"/>
+      <x:c r="AS159" s="66"/>
+      <x:c r="AZ159" s="66"/>
+      <x:c r="BF159" s="66"/>
+      <x:c r="BG159" s="66"/>
     </x:row>
     <x:row r="160" ht="15" hidden="0">
       <x:c r="A160" s="18"/>
@@ -6117,6 +8082,15 @@
       <x:c r="Y160" s="49"/>
       <x:c r="Z160" s="49"/>
       <x:c r="AA160" s="49"/>
+      <x:c r="AI160" s="66"/>
+      <x:c r="AK160" s="66"/>
+      <x:c r="AM160" s="66"/>
+      <x:c r="AO160" s="66"/>
+      <x:c r="AQ160" s="66"/>
+      <x:c r="AS160" s="66"/>
+      <x:c r="AZ160" s="66"/>
+      <x:c r="BF160" s="66"/>
+      <x:c r="BG160" s="66"/>
     </x:row>
     <x:row r="161" ht="15" hidden="0">
       <x:c r="A161" s="18"/>
@@ -6148,6 +8122,15 @@
       <x:c r="Y161" s="49"/>
       <x:c r="Z161" s="49"/>
       <x:c r="AA161" s="49"/>
+      <x:c r="AI161" s="66"/>
+      <x:c r="AK161" s="66"/>
+      <x:c r="AM161" s="66"/>
+      <x:c r="AO161" s="66"/>
+      <x:c r="AQ161" s="66"/>
+      <x:c r="AS161" s="66"/>
+      <x:c r="AZ161" s="66"/>
+      <x:c r="BF161" s="66"/>
+      <x:c r="BG161" s="66"/>
     </x:row>
     <x:row r="162" ht="15" hidden="0">
       <x:c r="A162" s="18"/>
@@ -6179,6 +8162,15 @@
       <x:c r="Y162" s="49"/>
       <x:c r="Z162" s="49"/>
       <x:c r="AA162" s="49"/>
+      <x:c r="AI162" s="66"/>
+      <x:c r="AK162" s="66"/>
+      <x:c r="AM162" s="66"/>
+      <x:c r="AO162" s="66"/>
+      <x:c r="AQ162" s="66"/>
+      <x:c r="AS162" s="66"/>
+      <x:c r="AZ162" s="66"/>
+      <x:c r="BF162" s="66"/>
+      <x:c r="BG162" s="66"/>
     </x:row>
     <x:row r="163" ht="15" hidden="0">
       <x:c r="A163" s="18"/>
@@ -6210,6 +8202,15 @@
       <x:c r="Y163" s="49"/>
       <x:c r="Z163" s="49"/>
       <x:c r="AA163" s="49"/>
+      <x:c r="AI163" s="66"/>
+      <x:c r="AK163" s="66"/>
+      <x:c r="AM163" s="66"/>
+      <x:c r="AO163" s="66"/>
+      <x:c r="AQ163" s="66"/>
+      <x:c r="AS163" s="66"/>
+      <x:c r="AZ163" s="66"/>
+      <x:c r="BF163" s="66"/>
+      <x:c r="BG163" s="66"/>
     </x:row>
     <x:row r="164" ht="15" hidden="0">
       <x:c r="A164" s="18"/>
@@ -6241,6 +8242,15 @@
       <x:c r="Y164" s="49"/>
       <x:c r="Z164" s="49"/>
       <x:c r="AA164" s="49"/>
+      <x:c r="AI164" s="66"/>
+      <x:c r="AK164" s="66"/>
+      <x:c r="AM164" s="66"/>
+      <x:c r="AO164" s="66"/>
+      <x:c r="AQ164" s="66"/>
+      <x:c r="AS164" s="66"/>
+      <x:c r="AZ164" s="66"/>
+      <x:c r="BF164" s="66"/>
+      <x:c r="BG164" s="66"/>
     </x:row>
     <x:row r="165" ht="15" hidden="0">
       <x:c r="A165" s="18"/>
@@ -6272,6 +8282,15 @@
       <x:c r="Y165" s="49"/>
       <x:c r="Z165" s="49"/>
       <x:c r="AA165" s="49"/>
+      <x:c r="AI165" s="66"/>
+      <x:c r="AK165" s="66"/>
+      <x:c r="AM165" s="66"/>
+      <x:c r="AO165" s="66"/>
+      <x:c r="AQ165" s="66"/>
+      <x:c r="AS165" s="66"/>
+      <x:c r="AZ165" s="66"/>
+      <x:c r="BF165" s="66"/>
+      <x:c r="BG165" s="66"/>
     </x:row>
     <x:row r="166" ht="15" hidden="0">
       <x:c r="A166" s="18"/>
@@ -6303,6 +8322,15 @@
       <x:c r="Y166" s="49"/>
       <x:c r="Z166" s="49"/>
       <x:c r="AA166" s="49"/>
+      <x:c r="AI166" s="66"/>
+      <x:c r="AK166" s="66"/>
+      <x:c r="AM166" s="66"/>
+      <x:c r="AO166" s="66"/>
+      <x:c r="AQ166" s="66"/>
+      <x:c r="AS166" s="66"/>
+      <x:c r="AZ166" s="66"/>
+      <x:c r="BF166" s="66"/>
+      <x:c r="BG166" s="66"/>
     </x:row>
     <x:row r="167" ht="15" hidden="0">
       <x:c r="A167" s="18"/>
@@ -6334,6 +8362,15 @@
       <x:c r="Y167" s="49"/>
       <x:c r="Z167" s="49"/>
       <x:c r="AA167" s="49"/>
+      <x:c r="AI167" s="66"/>
+      <x:c r="AK167" s="66"/>
+      <x:c r="AM167" s="66"/>
+      <x:c r="AO167" s="66"/>
+      <x:c r="AQ167" s="66"/>
+      <x:c r="AS167" s="66"/>
+      <x:c r="AZ167" s="66"/>
+      <x:c r="BF167" s="66"/>
+      <x:c r="BG167" s="66"/>
     </x:row>
     <x:row r="168" ht="15" hidden="0">
       <x:c r="A168" s="18"/>
@@ -6365,6 +8402,15 @@
       <x:c r="Y168" s="49"/>
       <x:c r="Z168" s="49"/>
       <x:c r="AA168" s="49"/>
+      <x:c r="AI168" s="66"/>
+      <x:c r="AK168" s="66"/>
+      <x:c r="AM168" s="66"/>
+      <x:c r="AO168" s="66"/>
+      <x:c r="AQ168" s="66"/>
+      <x:c r="AS168" s="66"/>
+      <x:c r="AZ168" s="66"/>
+      <x:c r="BF168" s="66"/>
+      <x:c r="BG168" s="66"/>
     </x:row>
     <x:row r="169" ht="15" hidden="0">
       <x:c r="A169" s="18"/>
@@ -6396,6 +8442,15 @@
       <x:c r="Y169" s="49"/>
       <x:c r="Z169" s="49"/>
       <x:c r="AA169" s="49"/>
+      <x:c r="AI169" s="66"/>
+      <x:c r="AK169" s="66"/>
+      <x:c r="AM169" s="66"/>
+      <x:c r="AO169" s="66"/>
+      <x:c r="AQ169" s="66"/>
+      <x:c r="AS169" s="66"/>
+      <x:c r="AZ169" s="66"/>
+      <x:c r="BF169" s="66"/>
+      <x:c r="BG169" s="66"/>
     </x:row>
     <x:row r="170" ht="15" hidden="0">
       <x:c r="A170" s="18"/>
@@ -6427,6 +8482,15 @@
       <x:c r="Y170" s="49"/>
       <x:c r="Z170" s="49"/>
       <x:c r="AA170" s="49"/>
+      <x:c r="AI170" s="66"/>
+      <x:c r="AK170" s="66"/>
+      <x:c r="AM170" s="66"/>
+      <x:c r="AO170" s="66"/>
+      <x:c r="AQ170" s="66"/>
+      <x:c r="AS170" s="66"/>
+      <x:c r="AZ170" s="66"/>
+      <x:c r="BF170" s="66"/>
+      <x:c r="BG170" s="66"/>
     </x:row>
     <x:row r="171" ht="15" hidden="0">
       <x:c r="A171" s="18"/>
@@ -6458,6 +8522,15 @@
       <x:c r="Y171" s="49"/>
       <x:c r="Z171" s="49"/>
       <x:c r="AA171" s="49"/>
+      <x:c r="AI171" s="66"/>
+      <x:c r="AK171" s="66"/>
+      <x:c r="AM171" s="66"/>
+      <x:c r="AO171" s="66"/>
+      <x:c r="AQ171" s="66"/>
+      <x:c r="AS171" s="66"/>
+      <x:c r="AZ171" s="66"/>
+      <x:c r="BF171" s="66"/>
+      <x:c r="BG171" s="66"/>
     </x:row>
     <x:row r="172" ht="15" hidden="0">
       <x:c r="A172" s="18"/>
@@ -6489,6 +8562,15 @@
       <x:c r="Y172" s="49"/>
       <x:c r="Z172" s="49"/>
       <x:c r="AA172" s="49"/>
+      <x:c r="AI172" s="66"/>
+      <x:c r="AK172" s="66"/>
+      <x:c r="AM172" s="66"/>
+      <x:c r="AO172" s="66"/>
+      <x:c r="AQ172" s="66"/>
+      <x:c r="AS172" s="66"/>
+      <x:c r="AZ172" s="66"/>
+      <x:c r="BF172" s="66"/>
+      <x:c r="BG172" s="66"/>
     </x:row>
     <x:row r="173" ht="15" hidden="0">
       <x:c r="A173" s="18"/>
@@ -6520,6 +8602,15 @@
       <x:c r="Y173" s="49"/>
       <x:c r="Z173" s="49"/>
       <x:c r="AA173" s="49"/>
+      <x:c r="AI173" s="66"/>
+      <x:c r="AK173" s="66"/>
+      <x:c r="AM173" s="66"/>
+      <x:c r="AO173" s="66"/>
+      <x:c r="AQ173" s="66"/>
+      <x:c r="AS173" s="66"/>
+      <x:c r="AZ173" s="66"/>
+      <x:c r="BF173" s="66"/>
+      <x:c r="BG173" s="66"/>
     </x:row>
     <x:row r="174" ht="15" hidden="0">
       <x:c r="A174" s="18"/>
@@ -6551,6 +8642,15 @@
       <x:c r="Y174" s="49"/>
       <x:c r="Z174" s="49"/>
       <x:c r="AA174" s="49"/>
+      <x:c r="AI174" s="66"/>
+      <x:c r="AK174" s="66"/>
+      <x:c r="AM174" s="66"/>
+      <x:c r="AO174" s="66"/>
+      <x:c r="AQ174" s="66"/>
+      <x:c r="AS174" s="66"/>
+      <x:c r="AZ174" s="66"/>
+      <x:c r="BF174" s="66"/>
+      <x:c r="BG174" s="66"/>
     </x:row>
     <x:row r="175" ht="15" hidden="0">
       <x:c r="A175" s="18"/>
@@ -6582,6 +8682,15 @@
       <x:c r="Y175" s="49"/>
       <x:c r="Z175" s="49"/>
       <x:c r="AA175" s="49"/>
+      <x:c r="AI175" s="66"/>
+      <x:c r="AK175" s="66"/>
+      <x:c r="AM175" s="66"/>
+      <x:c r="AO175" s="66"/>
+      <x:c r="AQ175" s="66"/>
+      <x:c r="AS175" s="66"/>
+      <x:c r="AZ175" s="66"/>
+      <x:c r="BF175" s="66"/>
+      <x:c r="BG175" s="66"/>
     </x:row>
     <x:row r="176" ht="15" hidden="0">
       <x:c r="A176" s="18"/>
@@ -6613,6 +8722,15 @@
       <x:c r="Y176" s="49"/>
       <x:c r="Z176" s="49"/>
       <x:c r="AA176" s="49"/>
+      <x:c r="AI176" s="66"/>
+      <x:c r="AK176" s="66"/>
+      <x:c r="AM176" s="66"/>
+      <x:c r="AO176" s="66"/>
+      <x:c r="AQ176" s="66"/>
+      <x:c r="AS176" s="66"/>
+      <x:c r="AZ176" s="66"/>
+      <x:c r="BF176" s="66"/>
+      <x:c r="BG176" s="66"/>
     </x:row>
     <x:row r="177" ht="15" hidden="0">
       <x:c r="A177" s="18"/>
@@ -6644,6 +8762,15 @@
       <x:c r="Y177" s="49"/>
       <x:c r="Z177" s="49"/>
       <x:c r="AA177" s="49"/>
+      <x:c r="AI177" s="66"/>
+      <x:c r="AK177" s="66"/>
+      <x:c r="AM177" s="66"/>
+      <x:c r="AO177" s="66"/>
+      <x:c r="AQ177" s="66"/>
+      <x:c r="AS177" s="66"/>
+      <x:c r="AZ177" s="66"/>
+      <x:c r="BF177" s="66"/>
+      <x:c r="BG177" s="66"/>
     </x:row>
     <x:row r="178" ht="15" hidden="0">
       <x:c r="A178" s="18"/>
@@ -6675,6 +8802,15 @@
       <x:c r="Y178" s="49"/>
       <x:c r="Z178" s="49"/>
       <x:c r="AA178" s="49"/>
+      <x:c r="AI178" s="66"/>
+      <x:c r="AK178" s="66"/>
+      <x:c r="AM178" s="66"/>
+      <x:c r="AO178" s="66"/>
+      <x:c r="AQ178" s="66"/>
+      <x:c r="AS178" s="66"/>
+      <x:c r="AZ178" s="66"/>
+      <x:c r="BF178" s="66"/>
+      <x:c r="BG178" s="66"/>
     </x:row>
     <x:row r="179" ht="15" hidden="0">
       <x:c r="A179" s="18"/>
@@ -6706,6 +8842,15 @@
       <x:c r="Y179" s="49"/>
       <x:c r="Z179" s="49"/>
       <x:c r="AA179" s="49"/>
+      <x:c r="AI179" s="66"/>
+      <x:c r="AK179" s="66"/>
+      <x:c r="AM179" s="66"/>
+      <x:c r="AO179" s="66"/>
+      <x:c r="AQ179" s="66"/>
+      <x:c r="AS179" s="66"/>
+      <x:c r="AZ179" s="66"/>
+      <x:c r="BF179" s="66"/>
+      <x:c r="BG179" s="66"/>
     </x:row>
     <x:row r="180" ht="15" hidden="0">
       <x:c r="A180" s="18"/>
@@ -6737,6 +8882,15 @@
       <x:c r="Y180" s="49"/>
       <x:c r="Z180" s="49"/>
       <x:c r="AA180" s="49"/>
+      <x:c r="AI180" s="66"/>
+      <x:c r="AK180" s="66"/>
+      <x:c r="AM180" s="66"/>
+      <x:c r="AO180" s="66"/>
+      <x:c r="AQ180" s="66"/>
+      <x:c r="AS180" s="66"/>
+      <x:c r="AZ180" s="66"/>
+      <x:c r="BF180" s="66"/>
+      <x:c r="BG180" s="66"/>
     </x:row>
     <x:row r="181" ht="15" hidden="0">
       <x:c r="A181" s="18"/>
@@ -6768,6 +8922,15 @@
       <x:c r="Y181" s="49"/>
       <x:c r="Z181" s="49"/>
       <x:c r="AA181" s="49"/>
+      <x:c r="AI181" s="66"/>
+      <x:c r="AK181" s="66"/>
+      <x:c r="AM181" s="66"/>
+      <x:c r="AO181" s="66"/>
+      <x:c r="AQ181" s="66"/>
+      <x:c r="AS181" s="66"/>
+      <x:c r="AZ181" s="66"/>
+      <x:c r="BF181" s="66"/>
+      <x:c r="BG181" s="66"/>
     </x:row>
     <x:row r="182" ht="15" hidden="0">
       <x:c r="A182" s="18"/>
@@ -6799,6 +8962,15 @@
       <x:c r="Y182" s="49"/>
       <x:c r="Z182" s="49"/>
       <x:c r="AA182" s="49"/>
+      <x:c r="AI182" s="66"/>
+      <x:c r="AK182" s="66"/>
+      <x:c r="AM182" s="66"/>
+      <x:c r="AO182" s="66"/>
+      <x:c r="AQ182" s="66"/>
+      <x:c r="AS182" s="66"/>
+      <x:c r="AZ182" s="66"/>
+      <x:c r="BF182" s="66"/>
+      <x:c r="BG182" s="66"/>
     </x:row>
     <x:row r="183" ht="15" hidden="0">
       <x:c r="A183" s="18"/>
@@ -6830,6 +9002,15 @@
       <x:c r="Y183" s="49"/>
       <x:c r="Z183" s="49"/>
       <x:c r="AA183" s="49"/>
+      <x:c r="AI183" s="66"/>
+      <x:c r="AK183" s="66"/>
+      <x:c r="AM183" s="66"/>
+      <x:c r="AO183" s="66"/>
+      <x:c r="AQ183" s="66"/>
+      <x:c r="AS183" s="66"/>
+      <x:c r="AZ183" s="66"/>
+      <x:c r="BF183" s="66"/>
+      <x:c r="BG183" s="66"/>
     </x:row>
     <x:row r="184" ht="15" hidden="0">
       <x:c r="A184" s="18"/>
@@ -6861,6 +9042,15 @@
       <x:c r="Y184" s="49"/>
       <x:c r="Z184" s="49"/>
       <x:c r="AA184" s="49"/>
+      <x:c r="AI184" s="66"/>
+      <x:c r="AK184" s="66"/>
+      <x:c r="AM184" s="66"/>
+      <x:c r="AO184" s="66"/>
+      <x:c r="AQ184" s="66"/>
+      <x:c r="AS184" s="66"/>
+      <x:c r="AZ184" s="66"/>
+      <x:c r="BF184" s="66"/>
+      <x:c r="BG184" s="66"/>
     </x:row>
     <x:row r="185" ht="15" hidden="0">
       <x:c r="A185" s="18"/>
@@ -6892,6 +9082,15 @@
       <x:c r="Y185" s="49"/>
       <x:c r="Z185" s="49"/>
       <x:c r="AA185" s="49"/>
+      <x:c r="AI185" s="66"/>
+      <x:c r="AK185" s="66"/>
+      <x:c r="AM185" s="66"/>
+      <x:c r="AO185" s="66"/>
+      <x:c r="AQ185" s="66"/>
+      <x:c r="AS185" s="66"/>
+      <x:c r="AZ185" s="66"/>
+      <x:c r="BF185" s="66"/>
+      <x:c r="BG185" s="66"/>
     </x:row>
     <x:row r="186" ht="15" hidden="0">
       <x:c r="A186" s="18"/>
@@ -6923,6 +9122,15 @@
       <x:c r="Y186" s="49"/>
       <x:c r="Z186" s="49"/>
       <x:c r="AA186" s="49"/>
+      <x:c r="AI186" s="66"/>
+      <x:c r="AK186" s="66"/>
+      <x:c r="AM186" s="66"/>
+      <x:c r="AO186" s="66"/>
+      <x:c r="AQ186" s="66"/>
+      <x:c r="AS186" s="66"/>
+      <x:c r="AZ186" s="66"/>
+      <x:c r="BF186" s="66"/>
+      <x:c r="BG186" s="66"/>
     </x:row>
     <x:row r="187" ht="15" hidden="0">
       <x:c r="A187" s="18"/>
@@ -6954,6 +9162,15 @@
       <x:c r="Y187" s="49"/>
       <x:c r="Z187" s="49"/>
       <x:c r="AA187" s="49"/>
+      <x:c r="AI187" s="66"/>
+      <x:c r="AK187" s="66"/>
+      <x:c r="AM187" s="66"/>
+      <x:c r="AO187" s="66"/>
+      <x:c r="AQ187" s="66"/>
+      <x:c r="AS187" s="66"/>
+      <x:c r="AZ187" s="66"/>
+      <x:c r="BF187" s="66"/>
+      <x:c r="BG187" s="66"/>
     </x:row>
     <x:row r="188" ht="15" hidden="0">
       <x:c r="A188" s="18"/>
@@ -6985,6 +9202,15 @@
       <x:c r="Y188" s="49"/>
       <x:c r="Z188" s="49"/>
       <x:c r="AA188" s="49"/>
+      <x:c r="AI188" s="66"/>
+      <x:c r="AK188" s="66"/>
+      <x:c r="AM188" s="66"/>
+      <x:c r="AO188" s="66"/>
+      <x:c r="AQ188" s="66"/>
+      <x:c r="AS188" s="66"/>
+      <x:c r="AZ188" s="66"/>
+      <x:c r="BF188" s="66"/>
+      <x:c r="BG188" s="66"/>
     </x:row>
     <x:row r="189" ht="15" hidden="0">
       <x:c r="A189" s="18"/>
@@ -7016,6 +9242,15 @@
       <x:c r="Y189" s="49"/>
       <x:c r="Z189" s="49"/>
       <x:c r="AA189" s="49"/>
+      <x:c r="AI189" s="66"/>
+      <x:c r="AK189" s="66"/>
+      <x:c r="AM189" s="66"/>
+      <x:c r="AO189" s="66"/>
+      <x:c r="AQ189" s="66"/>
+      <x:c r="AS189" s="66"/>
+      <x:c r="AZ189" s="66"/>
+      <x:c r="BF189" s="66"/>
+      <x:c r="BG189" s="66"/>
     </x:row>
     <x:row r="190" ht="15" hidden="0">
       <x:c r="A190" s="18"/>
@@ -7047,6 +9282,15 @@
       <x:c r="Y190" s="49"/>
       <x:c r="Z190" s="49"/>
       <x:c r="AA190" s="49"/>
+      <x:c r="AI190" s="66"/>
+      <x:c r="AK190" s="66"/>
+      <x:c r="AM190" s="66"/>
+      <x:c r="AO190" s="66"/>
+      <x:c r="AQ190" s="66"/>
+      <x:c r="AS190" s="66"/>
+      <x:c r="AZ190" s="66"/>
+      <x:c r="BF190" s="66"/>
+      <x:c r="BG190" s="66"/>
     </x:row>
     <x:row r="191" ht="15" hidden="0">
       <x:c r="A191" s="18"/>
@@ -7078,6 +9322,15 @@
       <x:c r="Y191" s="49"/>
       <x:c r="Z191" s="49"/>
       <x:c r="AA191" s="49"/>
+      <x:c r="AI191" s="66"/>
+      <x:c r="AK191" s="66"/>
+      <x:c r="AM191" s="66"/>
+      <x:c r="AO191" s="66"/>
+      <x:c r="AQ191" s="66"/>
+      <x:c r="AS191" s="66"/>
+      <x:c r="AZ191" s="66"/>
+      <x:c r="BF191" s="66"/>
+      <x:c r="BG191" s="66"/>
     </x:row>
     <x:row r="192" ht="15" hidden="0">
       <x:c r="A192" s="18"/>
@@ -7109,6 +9362,15 @@
       <x:c r="Y192" s="49"/>
       <x:c r="Z192" s="49"/>
       <x:c r="AA192" s="49"/>
+      <x:c r="AI192" s="66"/>
+      <x:c r="AK192" s="66"/>
+      <x:c r="AM192" s="66"/>
+      <x:c r="AO192" s="66"/>
+      <x:c r="AQ192" s="66"/>
+      <x:c r="AS192" s="66"/>
+      <x:c r="AZ192" s="66"/>
+      <x:c r="BF192" s="66"/>
+      <x:c r="BG192" s="66"/>
     </x:row>
     <x:row r="193" ht="15" hidden="0">
       <x:c r="A193" s="18"/>
@@ -7140,6 +9402,15 @@
       <x:c r="Y193" s="49"/>
       <x:c r="Z193" s="49"/>
       <x:c r="AA193" s="49"/>
+      <x:c r="AI193" s="66"/>
+      <x:c r="AK193" s="66"/>
+      <x:c r="AM193" s="66"/>
+      <x:c r="AO193" s="66"/>
+      <x:c r="AQ193" s="66"/>
+      <x:c r="AS193" s="66"/>
+      <x:c r="AZ193" s="66"/>
+      <x:c r="BF193" s="66"/>
+      <x:c r="BG193" s="66"/>
     </x:row>
     <x:row r="194" ht="15" hidden="0">
       <x:c r="A194" s="18"/>
@@ -7171,6 +9442,15 @@
       <x:c r="Y194" s="49"/>
       <x:c r="Z194" s="49"/>
       <x:c r="AA194" s="49"/>
+      <x:c r="AI194" s="66"/>
+      <x:c r="AK194" s="66"/>
+      <x:c r="AM194" s="66"/>
+      <x:c r="AO194" s="66"/>
+      <x:c r="AQ194" s="66"/>
+      <x:c r="AS194" s="66"/>
+      <x:c r="AZ194" s="66"/>
+      <x:c r="BF194" s="66"/>
+      <x:c r="BG194" s="66"/>
     </x:row>
     <x:row r="195" ht="15" hidden="0">
       <x:c r="A195" s="18"/>
@@ -7202,6 +9482,15 @@
       <x:c r="Y195" s="49"/>
       <x:c r="Z195" s="49"/>
       <x:c r="AA195" s="49"/>
+      <x:c r="AI195" s="66"/>
+      <x:c r="AK195" s="66"/>
+      <x:c r="AM195" s="66"/>
+      <x:c r="AO195" s="66"/>
+      <x:c r="AQ195" s="66"/>
+      <x:c r="AS195" s="66"/>
+      <x:c r="AZ195" s="66"/>
+      <x:c r="BF195" s="66"/>
+      <x:c r="BG195" s="66"/>
     </x:row>
     <x:row r="196" ht="15" hidden="0">
       <x:c r="A196" s="18"/>
@@ -7233,6 +9522,15 @@
       <x:c r="Y196" s="49"/>
       <x:c r="Z196" s="49"/>
       <x:c r="AA196" s="49"/>
+      <x:c r="AI196" s="66"/>
+      <x:c r="AK196" s="66"/>
+      <x:c r="AM196" s="66"/>
+      <x:c r="AO196" s="66"/>
+      <x:c r="AQ196" s="66"/>
+      <x:c r="AS196" s="66"/>
+      <x:c r="AZ196" s="66"/>
+      <x:c r="BF196" s="66"/>
+      <x:c r="BG196" s="66"/>
     </x:row>
     <x:row r="197" ht="15" hidden="0">
       <x:c r="A197" s="18"/>
@@ -7264,6 +9562,15 @@
       <x:c r="Y197" s="49"/>
       <x:c r="Z197" s="49"/>
       <x:c r="AA197" s="49"/>
+      <x:c r="AI197" s="66"/>
+      <x:c r="AK197" s="66"/>
+      <x:c r="AM197" s="66"/>
+      <x:c r="AO197" s="66"/>
+      <x:c r="AQ197" s="66"/>
+      <x:c r="AS197" s="66"/>
+      <x:c r="AZ197" s="66"/>
+      <x:c r="BF197" s="66"/>
+      <x:c r="BG197" s="66"/>
     </x:row>
     <x:row r="198" ht="15" hidden="0">
       <x:c r="A198" s="18"/>
@@ -7295,6 +9602,15 @@
       <x:c r="Y198" s="49"/>
       <x:c r="Z198" s="49"/>
       <x:c r="AA198" s="49"/>
+      <x:c r="AI198" s="66"/>
+      <x:c r="AK198" s="66"/>
+      <x:c r="AM198" s="66"/>
+      <x:c r="AO198" s="66"/>
+      <x:c r="AQ198" s="66"/>
+      <x:c r="AS198" s="66"/>
+      <x:c r="AZ198" s="66"/>
+      <x:c r="BF198" s="66"/>
+      <x:c r="BG198" s="66"/>
     </x:row>
     <x:row r="199" ht="15" hidden="0">
       <x:c r="A199" s="18"/>
@@ -7326,6 +9642,15 @@
       <x:c r="Y199" s="49"/>
       <x:c r="Z199" s="49"/>
       <x:c r="AA199" s="49"/>
+      <x:c r="AI199" s="66"/>
+      <x:c r="AK199" s="66"/>
+      <x:c r="AM199" s="66"/>
+      <x:c r="AO199" s="66"/>
+      <x:c r="AQ199" s="66"/>
+      <x:c r="AS199" s="66"/>
+      <x:c r="AZ199" s="66"/>
+      <x:c r="BF199" s="66"/>
+      <x:c r="BG199" s="66"/>
     </x:row>
     <x:row r="200" ht="15" hidden="0">
       <x:c r="A200" s="18"/>
@@ -7357,6 +9682,15 @@
       <x:c r="Y200" s="49"/>
       <x:c r="Z200" s="49"/>
       <x:c r="AA200" s="49"/>
+      <x:c r="AI200" s="66"/>
+      <x:c r="AK200" s="66"/>
+      <x:c r="AM200" s="66"/>
+      <x:c r="AO200" s="66"/>
+      <x:c r="AQ200" s="66"/>
+      <x:c r="AS200" s="66"/>
+      <x:c r="AZ200" s="66"/>
+      <x:c r="BF200" s="66"/>
+      <x:c r="BG200" s="66"/>
     </x:row>
     <x:row r="201" ht="15" hidden="0">
       <x:c r="A201" s="18"/>
@@ -7388,6 +9722,15 @@
       <x:c r="Y201" s="49"/>
       <x:c r="Z201" s="49"/>
       <x:c r="AA201" s="49"/>
+      <x:c r="AI201" s="66"/>
+      <x:c r="AK201" s="66"/>
+      <x:c r="AM201" s="66"/>
+      <x:c r="AO201" s="66"/>
+      <x:c r="AQ201" s="66"/>
+      <x:c r="AS201" s="66"/>
+      <x:c r="AZ201" s="66"/>
+      <x:c r="BF201" s="66"/>
+      <x:c r="BG201" s="66"/>
     </x:row>
     <x:row r="202">
       <x:c r="W202" s="49"/>
@@ -7481,6 +9824,121 @@
     <x:cfRule type="expression" dxfId="8" priority="5" aboveAverage="0" percent="0" bottom="0" rank="0" equalAverage="0">
       <x:formula>$Q2="high"</x:formula>
     </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AI2:AI201">
+    <x:cfRule type="cellIs" dxfId="9" priority="6" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="10" priority="7" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="11" priority="8" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AK2:AK201">
+    <x:cfRule type="cellIs" dxfId="12" priority="9" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="13" priority="10" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="14" priority="11" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AM2:AM201">
+    <x:cfRule type="cellIs" dxfId="15" priority="12" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="16" priority="13" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="17" priority="14" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AO2:AO201">
+    <x:cfRule type="cellIs" dxfId="18" priority="15" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="19" priority="16" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="20" priority="17" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AQ2:AQ201">
+    <x:cfRule type="cellIs" dxfId="21" priority="18" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="22" priority="19" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="23" priority="20" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AS2:AS201">
+    <x:cfRule type="cellIs" dxfId="24" priority="21" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="25" priority="22" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="26" priority="23" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AZ2:AZ201">
+    <x:cfRule type="cellIs" dxfId="27" priority="24" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="28" priority="25" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="29" priority="26" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="BF2:BF201">
+    <x:cfRule type="cellIs" dxfId="30" priority="27" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="31" priority="28" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="32" priority="29" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="BG2:BG201">
+    <x:cfRule type="cellIs" dxfId="33" priority="30" operator="greaterThanOrEqual">
+      <x:formula>0.8</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="34" priority="31" operator="between">
+      <x:formula>0.5</x:formula>
+      <x:formula>0.799999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="35" priority="32" operator="lessThan">
+      <x:formula>0.5</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="BD2:BD201">
+    <x:cfRule type="containsText" dxfId="36" priority="33" operator="containsText" text="Interesting"/>
+    <x:cfRule type="containsText" dxfId="37" priority="34" operator="containsText" text="Low Confidence"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="BE2:BE201">
+    <x:cfRule type="notContainsBlanks" dxfId="38" priority="35"/>
   </x:conditionalFormatting>
   <x:dataValidations count="7">
     <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="N2:N201">
@@ -10274,4 +12732,115 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="70" t="str">
+        <x:v>Collection Summary</x:v>
+      </x:c>
+      <x:c r="B1" s="71" t="str">
+        <x:v>AI-assisted findings; verify important identifications</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="74" t="str">
+        <x:v>Uploaded photographs</x:v>
+      </x:c>
+      <x:c r="B2" s="78"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="75" t="str">
+        <x:v>Detected stamps</x:v>
+      </x:c>
+      <x:c r="B3" s="79"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="75" t="str">
+        <x:v>Average confidence</x:v>
+      </x:c>
+      <x:c r="B4" s="81"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="75" t="str">
+        <x:v>Countries detected</x:v>
+      </x:c>
+      <x:c r="B5" s="79"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="75" t="str">
+        <x:v>Top countries</x:v>
+      </x:c>
+      <x:c r="B6" s="79"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="75" t="str">
+        <x:v>Themes detected</x:v>
+      </x:c>
+      <x:c r="B7" s="79"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="75" t="str">
+        <x:v>Top themes</x:v>
+      </x:c>
+      <x:c r="B8" s="79"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="75" t="str">
+        <x:v>Duplicate candidates</x:v>
+      </x:c>
+      <x:c r="B9" s="79"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="75" t="str">
+        <x:v>Unknown stamps</x:v>
+      </x:c>
+      <x:c r="B10" s="79"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="75" t="str">
+        <x:v>Low-quality images</x:v>
+      </x:c>
+      <x:c r="B11" s="79"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="75" t="str">
+        <x:v>Manual review count</x:v>
+      </x:c>
+      <x:c r="B12" s="79"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="75" t="str">
+        <x:v>Research candidates</x:v>
+      </x:c>
+      <x:c r="B13" s="79"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="75" t="str">
+        <x:v>Average image quality</x:v>
+      </x:c>
+      <x:c r="B14" s="81"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="75" t="str">
+        <x:v>Top recommendations</x:v>
+      </x:c>
+      <x:c r="B15" s="79"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="76" t="str">
+        <x:v>Processing time (seconds)</x:v>
+      </x:c>
+      <x:c r="B16" s="80"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>